<commit_message>
Add filter dropdown for control chart data points (10/25/50/100/All)
</commit_message>
<xml_diff>
--- a/SPC_Statistical_Calculator.xlsx
+++ b/SPC_Statistical_Calculator.xlsx
@@ -22,16 +22,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.00000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0000%"/>
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
-    <numFmt numFmtId="170" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="170" formatCode=";;;"/>
+    <numFmt numFmtId="171" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -132,6 +133,16 @@
       <b val="1"/>
       <color rgb="00047857"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00F97316"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00FFFFFF"/>
+      <sz val="1"/>
     </font>
   </fonts>
   <fills count="9">
@@ -254,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -360,6 +371,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -367,7 +385,7 @@
     <xf numFmtId="1" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -761,12 +779,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Charts'!$H$5:$H$54</f>
+              <f>'Charts'!$H$5:$H$104</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$I$5:$I$54</f>
+              <f>'Charts'!$I$5:$I$104</f>
             </numRef>
           </val>
         </ser>
@@ -796,12 +814,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Charts'!$H$5:$H$54</f>
+              <f>'Charts'!$H$5:$H$104</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$K$5:$K$54</f>
+              <f>'Charts'!$K$5:$K$104</f>
             </numRef>
           </val>
         </ser>
@@ -831,12 +849,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Charts'!$H$5:$H$54</f>
+              <f>'Charts'!$H$5:$H$104</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$L$5:$L$54</f>
+              <f>'Charts'!$L$5:$L$104</f>
             </numRef>
           </val>
         </ser>
@@ -866,12 +884,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Charts'!$H$5:$H$54</f>
+              <f>'Charts'!$H$5:$H$104</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$M$5:$M$54</f>
+              <f>'Charts'!$M$5:$M$104</f>
             </numRef>
           </val>
         </ser>
@@ -988,12 +1006,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Charts'!$H$5:$H$54</f>
+              <f>'Charts'!$H$5:$H$104</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$J$5:$J$54</f>
+              <f>'Charts'!$J$5:$J$104</f>
             </numRef>
           </val>
         </ser>
@@ -9577,7 +9595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:M54"/>
+  <dimension ref="B1:M104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9602,6 +9620,20 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="H2" s="43" t="inlineStr">
+        <is>
+          <t>Show Points:</t>
+        </is>
+      </c>
+      <c r="I2" s="44" t="n">
+        <v>50</v>
+      </c>
+      <c r="J2" s="45">
+        <f>IF(I2="All",1000,I2)</f>
+        <v/>
+      </c>
+    </row>
     <row r="3">
       <c r="B3" s="3" t="inlineStr">
         <is>
@@ -9613,7 +9645,7 @@
       <c r="E3" s="4" t="n"/>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>I-MR Control Chart Data (from Data Worksheet)</t>
+          <t>I-MR Control Chart Data (filtered by Show Points)</t>
         </is>
       </c>
       <c r="I3" s="4" t="n"/>
@@ -9675,1322 +9707,1322 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="43" t="n">
+      <c r="B5" s="46" t="n">
         <v>-4</v>
       </c>
-      <c r="C5" s="44">
+      <c r="C5" s="47">
         <f>Analysis!G9+B5*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D5" s="44">
+      <c r="D5" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B5^2),0)</f>
         <v/>
       </c>
-      <c r="E5" s="44">
+      <c r="E5" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C5-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H5" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="45">
-        <f>IF(Data!D5="""",NA(),Data!D5)</f>
-        <v/>
-      </c>
-      <c r="J5" s="45">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="K5" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L5" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M5" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I5" s="48">
+        <f>IF(OR(1&gt;$J$2,Data!D5=""),NA(),Data!D5)</f>
+        <v/>
+      </c>
+      <c r="J5" s="48">
+        <f>IF(1&gt;$J$2,NA(),NA())</f>
+        <v/>
+      </c>
+      <c r="K5" s="48">
+        <f>IF(OR(1&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L5" s="48">
+        <f>IF(OR(1&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M5" s="48">
+        <f>IF(OR(1&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="43" t="n">
+      <c r="B6" s="46" t="n">
         <v>-3.75</v>
       </c>
-      <c r="C6" s="44">
+      <c r="C6" s="47">
         <f>Analysis!G9+B6*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D6" s="44">
+      <c r="D6" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B6^2),0)</f>
         <v/>
       </c>
-      <c r="E6" s="44">
+      <c r="E6" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C6-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H6" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="I6" s="45">
-        <f>IF(Data!D6="""",NA(),Data!D6)</f>
-        <v/>
-      </c>
-      <c r="J6" s="45">
-        <f>IF(OR(Data!D6="""",Data!D5=""""),NA(),ABS(Data!D6-Data!D5))</f>
-        <v/>
-      </c>
-      <c r="K6" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L6" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M6" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I6" s="48">
+        <f>IF(OR(2&gt;$J$2,Data!D6=""),NA(),Data!D6)</f>
+        <v/>
+      </c>
+      <c r="J6" s="48">
+        <f>IF(OR(2&gt;$J$2,Data!D6="",Data!D5=""),NA(),ABS(Data!D6-Data!D5))</f>
+        <v/>
+      </c>
+      <c r="K6" s="48">
+        <f>IF(OR(2&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="48">
+        <f>IF(OR(2&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M6" s="48">
+        <f>IF(OR(2&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="43" t="n">
+      <c r="B7" s="46" t="n">
         <v>-3.5</v>
       </c>
-      <c r="C7" s="44">
+      <c r="C7" s="47">
         <f>Analysis!G9+B7*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D7" s="44">
+      <c r="D7" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B7^2),0)</f>
         <v/>
       </c>
-      <c r="E7" s="44">
+      <c r="E7" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C7-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H7" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="I7" s="45">
-        <f>IF(Data!D7="""",NA(),Data!D7)</f>
-        <v/>
-      </c>
-      <c r="J7" s="45">
-        <f>IF(OR(Data!D7="""",Data!D6=""""),NA(),ABS(Data!D7-Data!D6))</f>
-        <v/>
-      </c>
-      <c r="K7" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L7" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M7" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I7" s="48">
+        <f>IF(OR(3&gt;$J$2,Data!D7=""),NA(),Data!D7)</f>
+        <v/>
+      </c>
+      <c r="J7" s="48">
+        <f>IF(OR(3&gt;$J$2,Data!D7="",Data!D6=""),NA(),ABS(Data!D7-Data!D6))</f>
+        <v/>
+      </c>
+      <c r="K7" s="48">
+        <f>IF(OR(3&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L7" s="48">
+        <f>IF(OR(3&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M7" s="48">
+        <f>IF(OR(3&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="43" t="n">
+      <c r="B8" s="46" t="n">
         <v>-3.25</v>
       </c>
-      <c r="C8" s="44">
+      <c r="C8" s="47">
         <f>Analysis!G9+B8*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D8" s="44">
+      <c r="D8" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B8^2),0)</f>
         <v/>
       </c>
-      <c r="E8" s="44">
+      <c r="E8" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C8-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H8" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="I8" s="45">
-        <f>IF(Data!D8="""",NA(),Data!D8)</f>
-        <v/>
-      </c>
-      <c r="J8" s="45">
-        <f>IF(OR(Data!D8="""",Data!D7=""""),NA(),ABS(Data!D8-Data!D7))</f>
-        <v/>
-      </c>
-      <c r="K8" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L8" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M8" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I8" s="48">
+        <f>IF(OR(4&gt;$J$2,Data!D8=""),NA(),Data!D8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="48">
+        <f>IF(OR(4&gt;$J$2,Data!D8="",Data!D7=""),NA(),ABS(Data!D8-Data!D7))</f>
+        <v/>
+      </c>
+      <c r="K8" s="48">
+        <f>IF(OR(4&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L8" s="48">
+        <f>IF(OR(4&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M8" s="48">
+        <f>IF(OR(4&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="43" t="n">
+      <c r="B9" s="46" t="n">
         <v>-3</v>
       </c>
-      <c r="C9" s="44">
+      <c r="C9" s="47">
         <f>Analysis!G9+B9*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D9" s="44">
+      <c r="D9" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B9^2),0)</f>
         <v/>
       </c>
-      <c r="E9" s="44">
+      <c r="E9" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C9-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H9" s="36" t="n">
         <v>5</v>
       </c>
-      <c r="I9" s="45">
-        <f>IF(Data!D9="""",NA(),Data!D9)</f>
-        <v/>
-      </c>
-      <c r="J9" s="45">
-        <f>IF(OR(Data!D9="""",Data!D8=""""),NA(),ABS(Data!D9-Data!D8))</f>
-        <v/>
-      </c>
-      <c r="K9" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L9" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M9" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I9" s="48">
+        <f>IF(OR(5&gt;$J$2,Data!D9=""),NA(),Data!D9)</f>
+        <v/>
+      </c>
+      <c r="J9" s="48">
+        <f>IF(OR(5&gt;$J$2,Data!D9="",Data!D8=""),NA(),ABS(Data!D9-Data!D8))</f>
+        <v/>
+      </c>
+      <c r="K9" s="48">
+        <f>IF(OR(5&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L9" s="48">
+        <f>IF(OR(5&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M9" s="48">
+        <f>IF(OR(5&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="43" t="n">
+      <c r="B10" s="46" t="n">
         <v>-2.75</v>
       </c>
-      <c r="C10" s="44">
+      <c r="C10" s="47">
         <f>Analysis!G9+B10*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D10" s="44">
+      <c r="D10" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B10^2),0)</f>
         <v/>
       </c>
-      <c r="E10" s="44">
+      <c r="E10" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C10-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H10" s="36" t="n">
         <v>6</v>
       </c>
-      <c r="I10" s="45">
-        <f>IF(Data!D10="""",NA(),Data!D10)</f>
-        <v/>
-      </c>
-      <c r="J10" s="45">
-        <f>IF(OR(Data!D10="""",Data!D9=""""),NA(),ABS(Data!D10-Data!D9))</f>
-        <v/>
-      </c>
-      <c r="K10" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L10" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M10" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I10" s="48">
+        <f>IF(OR(6&gt;$J$2,Data!D10=""),NA(),Data!D10)</f>
+        <v/>
+      </c>
+      <c r="J10" s="48">
+        <f>IF(OR(6&gt;$J$2,Data!D10="",Data!D9=""),NA(),ABS(Data!D10-Data!D9))</f>
+        <v/>
+      </c>
+      <c r="K10" s="48">
+        <f>IF(OR(6&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L10" s="48">
+        <f>IF(OR(6&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M10" s="48">
+        <f>IF(OR(6&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="43" t="n">
+      <c r="B11" s="46" t="n">
         <v>-2.5</v>
       </c>
-      <c r="C11" s="44">
+      <c r="C11" s="47">
         <f>Analysis!G9+B11*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D11" s="44">
+      <c r="D11" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B11^2),0)</f>
         <v/>
       </c>
-      <c r="E11" s="44">
+      <c r="E11" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C11-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H11" s="36" t="n">
         <v>7</v>
       </c>
-      <c r="I11" s="45">
-        <f>IF(Data!D11="""",NA(),Data!D11)</f>
-        <v/>
-      </c>
-      <c r="J11" s="45">
-        <f>IF(OR(Data!D11="""",Data!D10=""""),NA(),ABS(Data!D11-Data!D10))</f>
-        <v/>
-      </c>
-      <c r="K11" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L11" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M11" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I11" s="48">
+        <f>IF(OR(7&gt;$J$2,Data!D11=""),NA(),Data!D11)</f>
+        <v/>
+      </c>
+      <c r="J11" s="48">
+        <f>IF(OR(7&gt;$J$2,Data!D11="",Data!D10=""),NA(),ABS(Data!D11-Data!D10))</f>
+        <v/>
+      </c>
+      <c r="K11" s="48">
+        <f>IF(OR(7&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L11" s="48">
+        <f>IF(OR(7&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M11" s="48">
+        <f>IF(OR(7&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="43" t="n">
+      <c r="B12" s="46" t="n">
         <v>-2.25</v>
       </c>
-      <c r="C12" s="44">
+      <c r="C12" s="47">
         <f>Analysis!G9+B12*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D12" s="44">
+      <c r="D12" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B12^2),0)</f>
         <v/>
       </c>
-      <c r="E12" s="44">
+      <c r="E12" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C12-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H12" s="36" t="n">
         <v>8</v>
       </c>
-      <c r="I12" s="45">
-        <f>IF(Data!D12="""",NA(),Data!D12)</f>
-        <v/>
-      </c>
-      <c r="J12" s="45">
-        <f>IF(OR(Data!D12="""",Data!D11=""""),NA(),ABS(Data!D12-Data!D11))</f>
-        <v/>
-      </c>
-      <c r="K12" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L12" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M12" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I12" s="48">
+        <f>IF(OR(8&gt;$J$2,Data!D12=""),NA(),Data!D12)</f>
+        <v/>
+      </c>
+      <c r="J12" s="48">
+        <f>IF(OR(8&gt;$J$2,Data!D12="",Data!D11=""),NA(),ABS(Data!D12-Data!D11))</f>
+        <v/>
+      </c>
+      <c r="K12" s="48">
+        <f>IF(OR(8&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L12" s="48">
+        <f>IF(OR(8&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M12" s="48">
+        <f>IF(OR(8&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="43" t="n">
+      <c r="B13" s="46" t="n">
         <v>-2</v>
       </c>
-      <c r="C13" s="44">
+      <c r="C13" s="47">
         <f>Analysis!G9+B13*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D13" s="44">
+      <c r="D13" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B13^2),0)</f>
         <v/>
       </c>
-      <c r="E13" s="44">
+      <c r="E13" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C13-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H13" s="36" t="n">
         <v>9</v>
       </c>
-      <c r="I13" s="45">
-        <f>IF(Data!D13="""",NA(),Data!D13)</f>
-        <v/>
-      </c>
-      <c r="J13" s="45">
-        <f>IF(OR(Data!D13="""",Data!D12=""""),NA(),ABS(Data!D13-Data!D12))</f>
-        <v/>
-      </c>
-      <c r="K13" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L13" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M13" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I13" s="48">
+        <f>IF(OR(9&gt;$J$2,Data!D13=""),NA(),Data!D13)</f>
+        <v/>
+      </c>
+      <c r="J13" s="48">
+        <f>IF(OR(9&gt;$J$2,Data!D13="",Data!D12=""),NA(),ABS(Data!D13-Data!D12))</f>
+        <v/>
+      </c>
+      <c r="K13" s="48">
+        <f>IF(OR(9&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L13" s="48">
+        <f>IF(OR(9&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M13" s="48">
+        <f>IF(OR(9&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="43" t="n">
+      <c r="B14" s="46" t="n">
         <v>-1.75</v>
       </c>
-      <c r="C14" s="44">
+      <c r="C14" s="47">
         <f>Analysis!G9+B14*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D14" s="44">
+      <c r="D14" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B14^2),0)</f>
         <v/>
       </c>
-      <c r="E14" s="44">
+      <c r="E14" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C14-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H14" s="36" t="n">
         <v>10</v>
       </c>
-      <c r="I14" s="45">
-        <f>IF(Data!D14="""",NA(),Data!D14)</f>
-        <v/>
-      </c>
-      <c r="J14" s="45">
-        <f>IF(OR(Data!D14="""",Data!D13=""""),NA(),ABS(Data!D14-Data!D13))</f>
-        <v/>
-      </c>
-      <c r="K14" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L14" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M14" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I14" s="48">
+        <f>IF(OR(10&gt;$J$2,Data!D14=""),NA(),Data!D14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="48">
+        <f>IF(OR(10&gt;$J$2,Data!D14="",Data!D13=""),NA(),ABS(Data!D14-Data!D13))</f>
+        <v/>
+      </c>
+      <c r="K14" s="48">
+        <f>IF(OR(10&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L14" s="48">
+        <f>IF(OR(10&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M14" s="48">
+        <f>IF(OR(10&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="43" t="n">
+      <c r="B15" s="46" t="n">
         <v>-1.5</v>
       </c>
-      <c r="C15" s="44">
+      <c r="C15" s="47">
         <f>Analysis!G9+B15*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D15" s="44">
+      <c r="D15" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B15^2),0)</f>
         <v/>
       </c>
-      <c r="E15" s="44">
+      <c r="E15" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C15-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H15" s="36" t="n">
         <v>11</v>
       </c>
-      <c r="I15" s="45">
-        <f>IF(Data!D15="""",NA(),Data!D15)</f>
-        <v/>
-      </c>
-      <c r="J15" s="45">
-        <f>IF(OR(Data!D15="""",Data!D14=""""),NA(),ABS(Data!D15-Data!D14))</f>
-        <v/>
-      </c>
-      <c r="K15" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L15" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M15" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I15" s="48">
+        <f>IF(OR(11&gt;$J$2,Data!D15=""),NA(),Data!D15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="48">
+        <f>IF(OR(11&gt;$J$2,Data!D15="",Data!D14=""),NA(),ABS(Data!D15-Data!D14))</f>
+        <v/>
+      </c>
+      <c r="K15" s="48">
+        <f>IF(OR(11&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L15" s="48">
+        <f>IF(OR(11&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M15" s="48">
+        <f>IF(OR(11&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="43" t="n">
+      <c r="B16" s="46" t="n">
         <v>-1.25</v>
       </c>
-      <c r="C16" s="44">
+      <c r="C16" s="47">
         <f>Analysis!G9+B16*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D16" s="44">
+      <c r="D16" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B16^2),0)</f>
         <v/>
       </c>
-      <c r="E16" s="44">
+      <c r="E16" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C16-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H16" s="36" t="n">
         <v>12</v>
       </c>
-      <c r="I16" s="45">
-        <f>IF(Data!D16="""",NA(),Data!D16)</f>
-        <v/>
-      </c>
-      <c r="J16" s="45">
-        <f>IF(OR(Data!D16="""",Data!D15=""""),NA(),ABS(Data!D16-Data!D15))</f>
-        <v/>
-      </c>
-      <c r="K16" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L16" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M16" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I16" s="48">
+        <f>IF(OR(12&gt;$J$2,Data!D16=""),NA(),Data!D16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="48">
+        <f>IF(OR(12&gt;$J$2,Data!D16="",Data!D15=""),NA(),ABS(Data!D16-Data!D15))</f>
+        <v/>
+      </c>
+      <c r="K16" s="48">
+        <f>IF(OR(12&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L16" s="48">
+        <f>IF(OR(12&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M16" s="48">
+        <f>IF(OR(12&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="43" t="n">
+      <c r="B17" s="46" t="n">
         <v>-1</v>
       </c>
-      <c r="C17" s="44">
+      <c r="C17" s="47">
         <f>Analysis!G9+B17*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D17" s="44">
+      <c r="D17" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B17^2),0)</f>
         <v/>
       </c>
-      <c r="E17" s="44">
+      <c r="E17" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C17-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H17" s="36" t="n">
         <v>13</v>
       </c>
-      <c r="I17" s="45">
-        <f>IF(Data!D17="""",NA(),Data!D17)</f>
-        <v/>
-      </c>
-      <c r="J17" s="45">
-        <f>IF(OR(Data!D17="""",Data!D16=""""),NA(),ABS(Data!D17-Data!D16))</f>
-        <v/>
-      </c>
-      <c r="K17" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L17" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M17" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I17" s="48">
+        <f>IF(OR(13&gt;$J$2,Data!D17=""),NA(),Data!D17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="48">
+        <f>IF(OR(13&gt;$J$2,Data!D17="",Data!D16=""),NA(),ABS(Data!D17-Data!D16))</f>
+        <v/>
+      </c>
+      <c r="K17" s="48">
+        <f>IF(OR(13&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L17" s="48">
+        <f>IF(OR(13&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M17" s="48">
+        <f>IF(OR(13&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="43" t="n">
+      <c r="B18" s="46" t="n">
         <v>-0.75</v>
       </c>
-      <c r="C18" s="44">
+      <c r="C18" s="47">
         <f>Analysis!G9+B18*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D18" s="44">
+      <c r="D18" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B18^2),0)</f>
         <v/>
       </c>
-      <c r="E18" s="44">
+      <c r="E18" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C18-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H18" s="36" t="n">
         <v>14</v>
       </c>
-      <c r="I18" s="45">
-        <f>IF(Data!D18="""",NA(),Data!D18)</f>
-        <v/>
-      </c>
-      <c r="J18" s="45">
-        <f>IF(OR(Data!D18="""",Data!D17=""""),NA(),ABS(Data!D18-Data!D17))</f>
-        <v/>
-      </c>
-      <c r="K18" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L18" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M18" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I18" s="48">
+        <f>IF(OR(14&gt;$J$2,Data!D18=""),NA(),Data!D18)</f>
+        <v/>
+      </c>
+      <c r="J18" s="48">
+        <f>IF(OR(14&gt;$J$2,Data!D18="",Data!D17=""),NA(),ABS(Data!D18-Data!D17))</f>
+        <v/>
+      </c>
+      <c r="K18" s="48">
+        <f>IF(OR(14&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L18" s="48">
+        <f>IF(OR(14&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M18" s="48">
+        <f>IF(OR(14&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="43" t="n">
+      <c r="B19" s="46" t="n">
         <v>-0.5</v>
       </c>
-      <c r="C19" s="44">
+      <c r="C19" s="47">
         <f>Analysis!G9+B19*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D19" s="44">
+      <c r="D19" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B19^2),0)</f>
         <v/>
       </c>
-      <c r="E19" s="44">
+      <c r="E19" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C19-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H19" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="I19" s="45">
-        <f>IF(Data!D19="""",NA(),Data!D19)</f>
-        <v/>
-      </c>
-      <c r="J19" s="45">
-        <f>IF(OR(Data!D19="""",Data!D18=""""),NA(),ABS(Data!D19-Data!D18))</f>
-        <v/>
-      </c>
-      <c r="K19" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L19" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M19" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I19" s="48">
+        <f>IF(OR(15&gt;$J$2,Data!D19=""),NA(),Data!D19)</f>
+        <v/>
+      </c>
+      <c r="J19" s="48">
+        <f>IF(OR(15&gt;$J$2,Data!D19="",Data!D18=""),NA(),ABS(Data!D19-Data!D18))</f>
+        <v/>
+      </c>
+      <c r="K19" s="48">
+        <f>IF(OR(15&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L19" s="48">
+        <f>IF(OR(15&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M19" s="48">
+        <f>IF(OR(15&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="43" t="n">
+      <c r="B20" s="46" t="n">
         <v>-0.25</v>
       </c>
-      <c r="C20" s="44">
+      <c r="C20" s="47">
         <f>Analysis!G9+B20*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D20" s="44">
+      <c r="D20" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B20^2),0)</f>
         <v/>
       </c>
-      <c r="E20" s="44">
+      <c r="E20" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C20-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H20" s="36" t="n">
         <v>16</v>
       </c>
-      <c r="I20" s="45">
-        <f>IF(Data!D20="""",NA(),Data!D20)</f>
-        <v/>
-      </c>
-      <c r="J20" s="45">
-        <f>IF(OR(Data!D20="""",Data!D19=""""),NA(),ABS(Data!D20-Data!D19))</f>
-        <v/>
-      </c>
-      <c r="K20" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L20" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M20" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I20" s="48">
+        <f>IF(OR(16&gt;$J$2,Data!D20=""),NA(),Data!D20)</f>
+        <v/>
+      </c>
+      <c r="J20" s="48">
+        <f>IF(OR(16&gt;$J$2,Data!D20="",Data!D19=""),NA(),ABS(Data!D20-Data!D19))</f>
+        <v/>
+      </c>
+      <c r="K20" s="48">
+        <f>IF(OR(16&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L20" s="48">
+        <f>IF(OR(16&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M20" s="48">
+        <f>IF(OR(16&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="43" t="n">
+      <c r="B21" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="C21" s="44">
+      <c r="C21" s="47">
         <f>Analysis!G9+B21*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D21" s="44">
+      <c r="D21" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B21^2),0)</f>
         <v/>
       </c>
-      <c r="E21" s="44">
+      <c r="E21" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C21-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H21" s="36" t="n">
         <v>17</v>
       </c>
-      <c r="I21" s="45">
-        <f>IF(Data!D21="""",NA(),Data!D21)</f>
-        <v/>
-      </c>
-      <c r="J21" s="45">
-        <f>IF(OR(Data!D21="""",Data!D20=""""),NA(),ABS(Data!D21-Data!D20))</f>
-        <v/>
-      </c>
-      <c r="K21" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L21" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M21" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I21" s="48">
+        <f>IF(OR(17&gt;$J$2,Data!D21=""),NA(),Data!D21)</f>
+        <v/>
+      </c>
+      <c r="J21" s="48">
+        <f>IF(OR(17&gt;$J$2,Data!D21="",Data!D20=""),NA(),ABS(Data!D21-Data!D20))</f>
+        <v/>
+      </c>
+      <c r="K21" s="48">
+        <f>IF(OR(17&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L21" s="48">
+        <f>IF(OR(17&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M21" s="48">
+        <f>IF(OR(17&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="43" t="n">
+      <c r="B22" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C22" s="44">
+      <c r="C22" s="47">
         <f>Analysis!G9+B22*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D22" s="44">
+      <c r="D22" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B22^2),0)</f>
         <v/>
       </c>
-      <c r="E22" s="44">
+      <c r="E22" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C22-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H22" s="36" t="n">
         <v>18</v>
       </c>
-      <c r="I22" s="45">
-        <f>IF(Data!D22="""",NA(),Data!D22)</f>
-        <v/>
-      </c>
-      <c r="J22" s="45">
-        <f>IF(OR(Data!D22="""",Data!D21=""""),NA(),ABS(Data!D22-Data!D21))</f>
-        <v/>
-      </c>
-      <c r="K22" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L22" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M22" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I22" s="48">
+        <f>IF(OR(18&gt;$J$2,Data!D22=""),NA(),Data!D22)</f>
+        <v/>
+      </c>
+      <c r="J22" s="48">
+        <f>IF(OR(18&gt;$J$2,Data!D22="",Data!D21=""),NA(),ABS(Data!D22-Data!D21))</f>
+        <v/>
+      </c>
+      <c r="K22" s="48">
+        <f>IF(OR(18&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L22" s="48">
+        <f>IF(OR(18&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M22" s="48">
+        <f>IF(OR(18&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="43" t="n">
+      <c r="B23" s="46" t="n">
         <v>0.5</v>
       </c>
-      <c r="C23" s="44">
+      <c r="C23" s="47">
         <f>Analysis!G9+B23*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D23" s="44">
+      <c r="D23" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B23^2),0)</f>
         <v/>
       </c>
-      <c r="E23" s="44">
+      <c r="E23" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C23-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H23" s="36" t="n">
         <v>19</v>
       </c>
-      <c r="I23" s="45">
-        <f>IF(Data!D23="""",NA(),Data!D23)</f>
-        <v/>
-      </c>
-      <c r="J23" s="45">
-        <f>IF(OR(Data!D23="""",Data!D22=""""),NA(),ABS(Data!D23-Data!D22))</f>
-        <v/>
-      </c>
-      <c r="K23" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L23" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M23" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I23" s="48">
+        <f>IF(OR(19&gt;$J$2,Data!D23=""),NA(),Data!D23)</f>
+        <v/>
+      </c>
+      <c r="J23" s="48">
+        <f>IF(OR(19&gt;$J$2,Data!D23="",Data!D22=""),NA(),ABS(Data!D23-Data!D22))</f>
+        <v/>
+      </c>
+      <c r="K23" s="48">
+        <f>IF(OR(19&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L23" s="48">
+        <f>IF(OR(19&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M23" s="48">
+        <f>IF(OR(19&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="43" t="n">
+      <c r="B24" s="46" t="n">
         <v>0.75</v>
       </c>
-      <c r="C24" s="44">
+      <c r="C24" s="47">
         <f>Analysis!G9+B24*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D24" s="44">
+      <c r="D24" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B24^2),0)</f>
         <v/>
       </c>
-      <c r="E24" s="44">
+      <c r="E24" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C24-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H24" s="36" t="n">
         <v>20</v>
       </c>
-      <c r="I24" s="45">
-        <f>IF(Data!D24="""",NA(),Data!D24)</f>
-        <v/>
-      </c>
-      <c r="J24" s="45">
-        <f>IF(OR(Data!D24="""",Data!D23=""""),NA(),ABS(Data!D24-Data!D23))</f>
-        <v/>
-      </c>
-      <c r="K24" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L24" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M24" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I24" s="48">
+        <f>IF(OR(20&gt;$J$2,Data!D24=""),NA(),Data!D24)</f>
+        <v/>
+      </c>
+      <c r="J24" s="48">
+        <f>IF(OR(20&gt;$J$2,Data!D24="",Data!D23=""),NA(),ABS(Data!D24-Data!D23))</f>
+        <v/>
+      </c>
+      <c r="K24" s="48">
+        <f>IF(OR(20&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L24" s="48">
+        <f>IF(OR(20&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M24" s="48">
+        <f>IF(OR(20&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="43" t="n">
+      <c r="B25" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="C25" s="44">
+      <c r="C25" s="47">
         <f>Analysis!G9+B25*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D25" s="44">
+      <c r="D25" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B25^2),0)</f>
         <v/>
       </c>
-      <c r="E25" s="44">
+      <c r="E25" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C25-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H25" s="36" t="n">
         <v>21</v>
       </c>
-      <c r="I25" s="45">
-        <f>IF(Data!D25="""",NA(),Data!D25)</f>
-        <v/>
-      </c>
-      <c r="J25" s="45">
-        <f>IF(OR(Data!D25="""",Data!D24=""""),NA(),ABS(Data!D25-Data!D24))</f>
-        <v/>
-      </c>
-      <c r="K25" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L25" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M25" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I25" s="48">
+        <f>IF(OR(21&gt;$J$2,Data!D25=""),NA(),Data!D25)</f>
+        <v/>
+      </c>
+      <c r="J25" s="48">
+        <f>IF(OR(21&gt;$J$2,Data!D25="",Data!D24=""),NA(),ABS(Data!D25-Data!D24))</f>
+        <v/>
+      </c>
+      <c r="K25" s="48">
+        <f>IF(OR(21&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L25" s="48">
+        <f>IF(OR(21&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M25" s="48">
+        <f>IF(OR(21&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="43" t="n">
+      <c r="B26" s="46" t="n">
         <v>1.25</v>
       </c>
-      <c r="C26" s="44">
+      <c r="C26" s="47">
         <f>Analysis!G9+B26*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D26" s="44">
+      <c r="D26" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B26^2),0)</f>
         <v/>
       </c>
-      <c r="E26" s="44">
+      <c r="E26" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C26-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H26" s="36" t="n">
         <v>22</v>
       </c>
-      <c r="I26" s="45">
-        <f>IF(Data!D26="""",NA(),Data!D26)</f>
-        <v/>
-      </c>
-      <c r="J26" s="45">
-        <f>IF(OR(Data!D26="""",Data!D25=""""),NA(),ABS(Data!D26-Data!D25))</f>
-        <v/>
-      </c>
-      <c r="K26" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L26" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M26" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I26" s="48">
+        <f>IF(OR(22&gt;$J$2,Data!D26=""),NA(),Data!D26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="48">
+        <f>IF(OR(22&gt;$J$2,Data!D26="",Data!D25=""),NA(),ABS(Data!D26-Data!D25))</f>
+        <v/>
+      </c>
+      <c r="K26" s="48">
+        <f>IF(OR(22&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L26" s="48">
+        <f>IF(OR(22&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M26" s="48">
+        <f>IF(OR(22&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="43" t="n">
+      <c r="B27" s="46" t="n">
         <v>1.5</v>
       </c>
-      <c r="C27" s="44">
+      <c r="C27" s="47">
         <f>Analysis!G9+B27*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D27" s="44">
+      <c r="D27" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B27^2),0)</f>
         <v/>
       </c>
-      <c r="E27" s="44">
+      <c r="E27" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C27-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H27" s="36" t="n">
         <v>23</v>
       </c>
-      <c r="I27" s="45">
-        <f>IF(Data!D27="""",NA(),Data!D27)</f>
-        <v/>
-      </c>
-      <c r="J27" s="45">
-        <f>IF(OR(Data!D27="""",Data!D26=""""),NA(),ABS(Data!D27-Data!D26))</f>
-        <v/>
-      </c>
-      <c r="K27" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L27" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M27" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I27" s="48">
+        <f>IF(OR(23&gt;$J$2,Data!D27=""),NA(),Data!D27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="48">
+        <f>IF(OR(23&gt;$J$2,Data!D27="",Data!D26=""),NA(),ABS(Data!D27-Data!D26))</f>
+        <v/>
+      </c>
+      <c r="K27" s="48">
+        <f>IF(OR(23&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L27" s="48">
+        <f>IF(OR(23&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M27" s="48">
+        <f>IF(OR(23&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="43" t="n">
+      <c r="B28" s="46" t="n">
         <v>1.75</v>
       </c>
-      <c r="C28" s="44">
+      <c r="C28" s="47">
         <f>Analysis!G9+B28*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D28" s="44">
+      <c r="D28" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B28^2),0)</f>
         <v/>
       </c>
-      <c r="E28" s="44">
+      <c r="E28" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C28-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H28" s="36" t="n">
         <v>24</v>
       </c>
-      <c r="I28" s="45">
-        <f>IF(Data!D28="""",NA(),Data!D28)</f>
-        <v/>
-      </c>
-      <c r="J28" s="45">
-        <f>IF(OR(Data!D28="""",Data!D27=""""),NA(),ABS(Data!D28-Data!D27))</f>
-        <v/>
-      </c>
-      <c r="K28" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L28" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M28" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I28" s="48">
+        <f>IF(OR(24&gt;$J$2,Data!D28=""),NA(),Data!D28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="48">
+        <f>IF(OR(24&gt;$J$2,Data!D28="",Data!D27=""),NA(),ABS(Data!D28-Data!D27))</f>
+        <v/>
+      </c>
+      <c r="K28" s="48">
+        <f>IF(OR(24&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L28" s="48">
+        <f>IF(OR(24&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M28" s="48">
+        <f>IF(OR(24&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="43" t="n">
+      <c r="B29" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="C29" s="44">
+      <c r="C29" s="47">
         <f>Analysis!G9+B29*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D29" s="44">
+      <c r="D29" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B29^2),0)</f>
         <v/>
       </c>
-      <c r="E29" s="44">
+      <c r="E29" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C29-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H29" s="36" t="n">
         <v>25</v>
       </c>
-      <c r="I29" s="45">
-        <f>IF(Data!D29="""",NA(),Data!D29)</f>
-        <v/>
-      </c>
-      <c r="J29" s="45">
-        <f>IF(OR(Data!D29="""",Data!D28=""""),NA(),ABS(Data!D29-Data!D28))</f>
-        <v/>
-      </c>
-      <c r="K29" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L29" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M29" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I29" s="48">
+        <f>IF(OR(25&gt;$J$2,Data!D29=""),NA(),Data!D29)</f>
+        <v/>
+      </c>
+      <c r="J29" s="48">
+        <f>IF(OR(25&gt;$J$2,Data!D29="",Data!D28=""),NA(),ABS(Data!D29-Data!D28))</f>
+        <v/>
+      </c>
+      <c r="K29" s="48">
+        <f>IF(OR(25&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L29" s="48">
+        <f>IF(OR(25&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M29" s="48">
+        <f>IF(OR(25&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="43" t="n">
+      <c r="B30" s="46" t="n">
         <v>2.25</v>
       </c>
-      <c r="C30" s="44">
+      <c r="C30" s="47">
         <f>Analysis!G9+B30*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D30" s="44">
+      <c r="D30" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B30^2),0)</f>
         <v/>
       </c>
-      <c r="E30" s="44">
+      <c r="E30" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C30-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H30" s="36" t="n">
         <v>26</v>
       </c>
-      <c r="I30" s="45">
-        <f>IF(Data!D30="""",NA(),Data!D30)</f>
-        <v/>
-      </c>
-      <c r="J30" s="45">
-        <f>IF(OR(Data!D30="""",Data!D29=""""),NA(),ABS(Data!D30-Data!D29))</f>
-        <v/>
-      </c>
-      <c r="K30" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L30" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M30" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I30" s="48">
+        <f>IF(OR(26&gt;$J$2,Data!D30=""),NA(),Data!D30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="48">
+        <f>IF(OR(26&gt;$J$2,Data!D30="",Data!D29=""),NA(),ABS(Data!D30-Data!D29))</f>
+        <v/>
+      </c>
+      <c r="K30" s="48">
+        <f>IF(OR(26&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L30" s="48">
+        <f>IF(OR(26&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M30" s="48">
+        <f>IF(OR(26&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="43" t="n">
+      <c r="B31" s="46" t="n">
         <v>2.5</v>
       </c>
-      <c r="C31" s="44">
+      <c r="C31" s="47">
         <f>Analysis!G9+B31*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D31" s="44">
+      <c r="D31" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B31^2),0)</f>
         <v/>
       </c>
-      <c r="E31" s="44">
+      <c r="E31" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C31-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H31" s="36" t="n">
         <v>27</v>
       </c>
-      <c r="I31" s="45">
-        <f>IF(Data!D31="""",NA(),Data!D31)</f>
-        <v/>
-      </c>
-      <c r="J31" s="45">
-        <f>IF(OR(Data!D31="""",Data!D30=""""),NA(),ABS(Data!D31-Data!D30))</f>
-        <v/>
-      </c>
-      <c r="K31" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L31" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M31" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I31" s="48">
+        <f>IF(OR(27&gt;$J$2,Data!D31=""),NA(),Data!D31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="48">
+        <f>IF(OR(27&gt;$J$2,Data!D31="",Data!D30=""),NA(),ABS(Data!D31-Data!D30))</f>
+        <v/>
+      </c>
+      <c r="K31" s="48">
+        <f>IF(OR(27&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L31" s="48">
+        <f>IF(OR(27&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M31" s="48">
+        <f>IF(OR(27&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="43" t="n">
+      <c r="B32" s="46" t="n">
         <v>2.75</v>
       </c>
-      <c r="C32" s="44">
+      <c r="C32" s="47">
         <f>Analysis!G9+B32*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D32" s="44">
+      <c r="D32" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B32^2),0)</f>
         <v/>
       </c>
-      <c r="E32" s="44">
+      <c r="E32" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C32-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H32" s="36" t="n">
         <v>28</v>
       </c>
-      <c r="I32" s="45">
-        <f>IF(Data!D32="""",NA(),Data!D32)</f>
-        <v/>
-      </c>
-      <c r="J32" s="45">
-        <f>IF(OR(Data!D32="""",Data!D31=""""),NA(),ABS(Data!D32-Data!D31))</f>
-        <v/>
-      </c>
-      <c r="K32" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L32" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M32" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I32" s="48">
+        <f>IF(OR(28&gt;$J$2,Data!D32=""),NA(),Data!D32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="48">
+        <f>IF(OR(28&gt;$J$2,Data!D32="",Data!D31=""),NA(),ABS(Data!D32-Data!D31))</f>
+        <v/>
+      </c>
+      <c r="K32" s="48">
+        <f>IF(OR(28&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L32" s="48">
+        <f>IF(OR(28&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M32" s="48">
+        <f>IF(OR(28&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="43" t="n">
+      <c r="B33" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="C33" s="44">
+      <c r="C33" s="47">
         <f>Analysis!G9+B33*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D33" s="44">
+      <c r="D33" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B33^2),0)</f>
         <v/>
       </c>
-      <c r="E33" s="44">
+      <c r="E33" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C33-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H33" s="36" t="n">
         <v>29</v>
       </c>
-      <c r="I33" s="45">
-        <f>IF(Data!D33="""",NA(),Data!D33)</f>
-        <v/>
-      </c>
-      <c r="J33" s="45">
-        <f>IF(OR(Data!D33="""",Data!D32=""""),NA(),ABS(Data!D33-Data!D32))</f>
-        <v/>
-      </c>
-      <c r="K33" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L33" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M33" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I33" s="48">
+        <f>IF(OR(29&gt;$J$2,Data!D33=""),NA(),Data!D33)</f>
+        <v/>
+      </c>
+      <c r="J33" s="48">
+        <f>IF(OR(29&gt;$J$2,Data!D33="",Data!D32=""),NA(),ABS(Data!D33-Data!D32))</f>
+        <v/>
+      </c>
+      <c r="K33" s="48">
+        <f>IF(OR(29&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L33" s="48">
+        <f>IF(OR(29&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M33" s="48">
+        <f>IF(OR(29&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="43" t="n">
+      <c r="B34" s="46" t="n">
         <v>3.25</v>
       </c>
-      <c r="C34" s="44">
+      <c r="C34" s="47">
         <f>Analysis!G9+B34*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D34" s="44">
+      <c r="D34" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B34^2),0)</f>
         <v/>
       </c>
-      <c r="E34" s="44">
+      <c r="E34" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C34-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H34" s="36" t="n">
         <v>30</v>
       </c>
-      <c r="I34" s="45">
-        <f>IF(Data!D34="""",NA(),Data!D34)</f>
-        <v/>
-      </c>
-      <c r="J34" s="45">
-        <f>IF(OR(Data!D34="""",Data!D33=""""),NA(),ABS(Data!D34-Data!D33))</f>
-        <v/>
-      </c>
-      <c r="K34" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L34" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M34" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I34" s="48">
+        <f>IF(OR(30&gt;$J$2,Data!D34=""),NA(),Data!D34)</f>
+        <v/>
+      </c>
+      <c r="J34" s="48">
+        <f>IF(OR(30&gt;$J$2,Data!D34="",Data!D33=""),NA(),ABS(Data!D34-Data!D33))</f>
+        <v/>
+      </c>
+      <c r="K34" s="48">
+        <f>IF(OR(30&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L34" s="48">
+        <f>IF(OR(30&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M34" s="48">
+        <f>IF(OR(30&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="43" t="n">
+      <c r="B35" s="46" t="n">
         <v>3.5</v>
       </c>
-      <c r="C35" s="44">
+      <c r="C35" s="47">
         <f>Analysis!G9+B35*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D35" s="44">
+      <c r="D35" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B35^2),0)</f>
         <v/>
       </c>
-      <c r="E35" s="44">
+      <c r="E35" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C35-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H35" s="36" t="n">
         <v>31</v>
       </c>
-      <c r="I35" s="45">
-        <f>IF(Data!D35="""",NA(),Data!D35)</f>
-        <v/>
-      </c>
-      <c r="J35" s="45">
-        <f>IF(OR(Data!D35="""",Data!D34=""""),NA(),ABS(Data!D35-Data!D34))</f>
-        <v/>
-      </c>
-      <c r="K35" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L35" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M35" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I35" s="48">
+        <f>IF(OR(31&gt;$J$2,Data!D35=""),NA(),Data!D35)</f>
+        <v/>
+      </c>
+      <c r="J35" s="48">
+        <f>IF(OR(31&gt;$J$2,Data!D35="",Data!D34=""),NA(),ABS(Data!D35-Data!D34))</f>
+        <v/>
+      </c>
+      <c r="K35" s="48">
+        <f>IF(OR(31&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L35" s="48">
+        <f>IF(OR(31&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M35" s="48">
+        <f>IF(OR(31&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="43" t="n">
+      <c r="B36" s="46" t="n">
         <v>3.75</v>
       </c>
-      <c r="C36" s="44">
+      <c r="C36" s="47">
         <f>Analysis!G9+B36*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D36" s="44">
+      <c r="D36" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B36^2),0)</f>
         <v/>
       </c>
-      <c r="E36" s="44">
+      <c r="E36" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C36-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H36" s="36" t="n">
         <v>32</v>
       </c>
-      <c r="I36" s="45">
-        <f>IF(Data!D36="""",NA(),Data!D36)</f>
-        <v/>
-      </c>
-      <c r="J36" s="45">
-        <f>IF(OR(Data!D36="""",Data!D35=""""),NA(),ABS(Data!D36-Data!D35))</f>
-        <v/>
-      </c>
-      <c r="K36" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L36" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M36" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I36" s="48">
+        <f>IF(OR(32&gt;$J$2,Data!D36=""),NA(),Data!D36)</f>
+        <v/>
+      </c>
+      <c r="J36" s="48">
+        <f>IF(OR(32&gt;$J$2,Data!D36="",Data!D35=""),NA(),ABS(Data!D36-Data!D35))</f>
+        <v/>
+      </c>
+      <c r="K36" s="48">
+        <f>IF(OR(32&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L36" s="48">
+        <f>IF(OR(32&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M36" s="48">
+        <f>IF(OR(32&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="43" t="n">
+      <c r="B37" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="C37" s="44">
+      <c r="C37" s="47">
         <f>Analysis!G9+B37*Analysis!G10</f>
         <v/>
       </c>
-      <c r="D37" s="44">
+      <c r="D37" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*B37^2),0)</f>
         <v/>
       </c>
-      <c r="E37" s="44">
+      <c r="E37" s="47">
         <f>IF(Analysis!G10&gt;0,(1/(Analysis!G10*SQRT(2*PI())))*EXP(-0.5*((C37-Analysis!C6)/Analysis!G10)^2),0)</f>
         <v/>
       </c>
       <c r="H37" s="36" t="n">
         <v>33</v>
       </c>
-      <c r="I37" s="45">
-        <f>IF(Data!D37="""",NA(),Data!D37)</f>
-        <v/>
-      </c>
-      <c r="J37" s="45">
-        <f>IF(OR(Data!D37="""",Data!D36=""""),NA(),ABS(Data!D37-Data!D36))</f>
-        <v/>
-      </c>
-      <c r="K37" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L37" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M37" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I37" s="48">
+        <f>IF(OR(33&gt;$J$2,Data!D37=""),NA(),Data!D37)</f>
+        <v/>
+      </c>
+      <c r="J37" s="48">
+        <f>IF(OR(33&gt;$J$2,Data!D37="",Data!D36=""),NA(),ABS(Data!D37-Data!D36))</f>
+        <v/>
+      </c>
+      <c r="K37" s="48">
+        <f>IF(OR(33&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L37" s="48">
+        <f>IF(OR(33&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M37" s="48">
+        <f>IF(OR(33&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -10998,24 +11030,24 @@
       <c r="H38" s="36" t="n">
         <v>34</v>
       </c>
-      <c r="I38" s="45">
-        <f>IF(Data!D38="""",NA(),Data!D38)</f>
-        <v/>
-      </c>
-      <c r="J38" s="45">
-        <f>IF(OR(Data!D38="""",Data!D37=""""),NA(),ABS(Data!D38-Data!D37))</f>
-        <v/>
-      </c>
-      <c r="K38" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L38" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M38" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I38" s="48">
+        <f>IF(OR(34&gt;$J$2,Data!D38=""),NA(),Data!D38)</f>
+        <v/>
+      </c>
+      <c r="J38" s="48">
+        <f>IF(OR(34&gt;$J$2,Data!D38="",Data!D37=""),NA(),ABS(Data!D38-Data!D37))</f>
+        <v/>
+      </c>
+      <c r="K38" s="48">
+        <f>IF(OR(34&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L38" s="48">
+        <f>IF(OR(34&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M38" s="48">
+        <f>IF(OR(34&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11023,24 +11055,24 @@
       <c r="H39" s="36" t="n">
         <v>35</v>
       </c>
-      <c r="I39" s="45">
-        <f>IF(Data!D39="""",NA(),Data!D39)</f>
-        <v/>
-      </c>
-      <c r="J39" s="45">
-        <f>IF(OR(Data!D39="""",Data!D38=""""),NA(),ABS(Data!D39-Data!D38))</f>
-        <v/>
-      </c>
-      <c r="K39" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L39" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M39" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I39" s="48">
+        <f>IF(OR(35&gt;$J$2,Data!D39=""),NA(),Data!D39)</f>
+        <v/>
+      </c>
+      <c r="J39" s="48">
+        <f>IF(OR(35&gt;$J$2,Data!D39="",Data!D38=""),NA(),ABS(Data!D39-Data!D38))</f>
+        <v/>
+      </c>
+      <c r="K39" s="48">
+        <f>IF(OR(35&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L39" s="48">
+        <f>IF(OR(35&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M39" s="48">
+        <f>IF(OR(35&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11056,24 +11088,24 @@
       <c r="H40" s="36" t="n">
         <v>36</v>
       </c>
-      <c r="I40" s="45">
-        <f>IF(Data!D40="""",NA(),Data!D40)</f>
-        <v/>
-      </c>
-      <c r="J40" s="45">
-        <f>IF(OR(Data!D40="""",Data!D39=""""),NA(),ABS(Data!D40-Data!D39))</f>
-        <v/>
-      </c>
-      <c r="K40" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L40" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M40" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I40" s="48">
+        <f>IF(OR(36&gt;$J$2,Data!D40=""),NA(),Data!D40)</f>
+        <v/>
+      </c>
+      <c r="J40" s="48">
+        <f>IF(OR(36&gt;$J$2,Data!D40="",Data!D39=""),NA(),ABS(Data!D40-Data!D39))</f>
+        <v/>
+      </c>
+      <c r="K40" s="48">
+        <f>IF(OR(36&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L40" s="48">
+        <f>IF(OR(36&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M40" s="48">
+        <f>IF(OR(36&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11101,106 +11133,106 @@
       <c r="H41" s="36" t="n">
         <v>37</v>
       </c>
-      <c r="I41" s="45">
-        <f>IF(Data!D41="""",NA(),Data!D41)</f>
-        <v/>
-      </c>
-      <c r="J41" s="45">
-        <f>IF(OR(Data!D41="""",Data!D40=""""),NA(),ABS(Data!D41-Data!D40))</f>
-        <v/>
-      </c>
-      <c r="K41" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L41" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M41" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I41" s="48">
+        <f>IF(OR(37&gt;$J$2,Data!D41=""),NA(),Data!D41)</f>
+        <v/>
+      </c>
+      <c r="J41" s="48">
+        <f>IF(OR(37&gt;$J$2,Data!D41="",Data!D40=""),NA(),ABS(Data!D41-Data!D40))</f>
+        <v/>
+      </c>
+      <c r="K41" s="48">
+        <f>IF(OR(37&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L41" s="48">
+        <f>IF(OR(37&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M41" s="48">
+        <f>IF(OR(37&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="46" t="inlineStr">
+      <c r="B42" s="49" t="inlineStr">
         <is>
           <t>Cp</t>
         </is>
       </c>
-      <c r="C42" s="43">
+      <c r="C42" s="46">
         <f>Analysis!G17</f>
         <v/>
       </c>
-      <c r="D42" s="43">
+      <c r="D42" s="46">
         <f>Analysis!C16</f>
         <v/>
       </c>
-      <c r="E42" s="43" t="n">
+      <c r="E42" s="46" t="n">
         <v>1</v>
       </c>
       <c r="H42" s="36" t="n">
         <v>38</v>
       </c>
-      <c r="I42" s="45">
-        <f>IF(Data!D42="""",NA(),Data!D42)</f>
-        <v/>
-      </c>
-      <c r="J42" s="45">
-        <f>IF(OR(Data!D42="""",Data!D41=""""),NA(),ABS(Data!D42-Data!D41))</f>
-        <v/>
-      </c>
-      <c r="K42" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L42" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M42" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I42" s="48">
+        <f>IF(OR(38&gt;$J$2,Data!D42=""),NA(),Data!D42)</f>
+        <v/>
+      </c>
+      <c r="J42" s="48">
+        <f>IF(OR(38&gt;$J$2,Data!D42="",Data!D41=""),NA(),ABS(Data!D42-Data!D41))</f>
+        <v/>
+      </c>
+      <c r="K42" s="48">
+        <f>IF(OR(38&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L42" s="48">
+        <f>IF(OR(38&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M42" s="48">
+        <f>IF(OR(38&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="46" t="inlineStr">
+      <c r="B43" s="49" t="inlineStr">
         <is>
           <t>Cpk</t>
         </is>
       </c>
-      <c r="C43" s="43">
+      <c r="C43" s="46">
         <f>Analysis!G18</f>
         <v/>
       </c>
-      <c r="D43" s="43">
+      <c r="D43" s="46">
         <f>Analysis!C16</f>
         <v/>
       </c>
-      <c r="E43" s="43" t="n">
+      <c r="E43" s="46" t="n">
         <v>1</v>
       </c>
       <c r="H43" s="36" t="n">
         <v>39</v>
       </c>
-      <c r="I43" s="45">
-        <f>IF(Data!D43="""",NA(),Data!D43)</f>
-        <v/>
-      </c>
-      <c r="J43" s="45">
-        <f>IF(OR(Data!D43="""",Data!D42=""""),NA(),ABS(Data!D43-Data!D42))</f>
-        <v/>
-      </c>
-      <c r="K43" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L43" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M43" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I43" s="48">
+        <f>IF(OR(39&gt;$J$2,Data!D43=""),NA(),Data!D43)</f>
+        <v/>
+      </c>
+      <c r="J43" s="48">
+        <f>IF(OR(39&gt;$J$2,Data!D43="",Data!D42=""),NA(),ABS(Data!D43-Data!D42))</f>
+        <v/>
+      </c>
+      <c r="K43" s="48">
+        <f>IF(OR(39&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L43" s="48">
+        <f>IF(OR(39&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M43" s="48">
+        <f>IF(OR(39&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11208,24 +11240,24 @@
       <c r="H44" s="36" t="n">
         <v>40</v>
       </c>
-      <c r="I44" s="45">
-        <f>IF(Data!D44="""",NA(),Data!D44)</f>
-        <v/>
-      </c>
-      <c r="J44" s="45">
-        <f>IF(OR(Data!D44="""",Data!D43=""""),NA(),ABS(Data!D44-Data!D43))</f>
-        <v/>
-      </c>
-      <c r="K44" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L44" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M44" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I44" s="48">
+        <f>IF(OR(40&gt;$J$2,Data!D44=""),NA(),Data!D44)</f>
+        <v/>
+      </c>
+      <c r="J44" s="48">
+        <f>IF(OR(40&gt;$J$2,Data!D44="",Data!D43=""),NA(),ABS(Data!D44-Data!D43))</f>
+        <v/>
+      </c>
+      <c r="K44" s="48">
+        <f>IF(OR(40&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L44" s="48">
+        <f>IF(OR(40&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M44" s="48">
+        <f>IF(OR(40&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11233,24 +11265,24 @@
       <c r="H45" s="36" t="n">
         <v>41</v>
       </c>
-      <c r="I45" s="45">
-        <f>IF(Data!D45="""",NA(),Data!D45)</f>
-        <v/>
-      </c>
-      <c r="J45" s="45">
-        <f>IF(OR(Data!D45="""",Data!D44=""""),NA(),ABS(Data!D45-Data!D44))</f>
-        <v/>
-      </c>
-      <c r="K45" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L45" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M45" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I45" s="48">
+        <f>IF(OR(41&gt;$J$2,Data!D45=""),NA(),Data!D45)</f>
+        <v/>
+      </c>
+      <c r="J45" s="48">
+        <f>IF(OR(41&gt;$J$2,Data!D45="",Data!D44=""),NA(),ABS(Data!D45-Data!D44))</f>
+        <v/>
+      </c>
+      <c r="K45" s="48">
+        <f>IF(OR(41&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L45" s="48">
+        <f>IF(OR(41&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M45" s="48">
+        <f>IF(OR(41&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11266,24 +11298,24 @@
       <c r="H46" s="36" t="n">
         <v>42</v>
       </c>
-      <c r="I46" s="45">
-        <f>IF(Data!D46="""",NA(),Data!D46)</f>
-        <v/>
-      </c>
-      <c r="J46" s="45">
-        <f>IF(OR(Data!D46="""",Data!D45=""""),NA(),ABS(Data!D46-Data!D45))</f>
-        <v/>
-      </c>
-      <c r="K46" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L46" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M46" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I46" s="48">
+        <f>IF(OR(42&gt;$J$2,Data!D46=""),NA(),Data!D46)</f>
+        <v/>
+      </c>
+      <c r="J46" s="48">
+        <f>IF(OR(42&gt;$J$2,Data!D46="",Data!D45=""),NA(),ABS(Data!D46-Data!D45))</f>
+        <v/>
+      </c>
+      <c r="K46" s="48">
+        <f>IF(OR(42&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L46" s="48">
+        <f>IF(OR(42&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M46" s="48">
+        <f>IF(OR(42&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11309,24 +11341,24 @@
       <c r="H47" s="36" t="n">
         <v>43</v>
       </c>
-      <c r="I47" s="45">
-        <f>IF(Data!D47="""",NA(),Data!D47)</f>
-        <v/>
-      </c>
-      <c r="J47" s="45">
-        <f>IF(OR(Data!D47="""",Data!D46=""""),NA(),ABS(Data!D47-Data!D46))</f>
-        <v/>
-      </c>
-      <c r="K47" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L47" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M47" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I47" s="48">
+        <f>IF(OR(43&gt;$J$2,Data!D47=""),NA(),Data!D47)</f>
+        <v/>
+      </c>
+      <c r="J47" s="48">
+        <f>IF(OR(43&gt;$J$2,Data!D47="",Data!D46=""),NA(),ABS(Data!D47-Data!D46))</f>
+        <v/>
+      </c>
+      <c r="K47" s="48">
+        <f>IF(OR(43&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L47" s="48">
+        <f>IF(OR(43&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M47" s="48">
+        <f>IF(OR(43&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11352,24 +11384,24 @@
       <c r="H48" s="36" t="n">
         <v>44</v>
       </c>
-      <c r="I48" s="45">
-        <f>IF(Data!D48="""",NA(),Data!D48)</f>
-        <v/>
-      </c>
-      <c r="J48" s="45">
-        <f>IF(OR(Data!D48="""",Data!D47=""""),NA(),ABS(Data!D48-Data!D47))</f>
-        <v/>
-      </c>
-      <c r="K48" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L48" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M48" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I48" s="48">
+        <f>IF(OR(44&gt;$J$2,Data!D48=""),NA(),Data!D48)</f>
+        <v/>
+      </c>
+      <c r="J48" s="48">
+        <f>IF(OR(44&gt;$J$2,Data!D48="",Data!D47=""),NA(),ABS(Data!D48-Data!D47))</f>
+        <v/>
+      </c>
+      <c r="K48" s="48">
+        <f>IF(OR(44&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L48" s="48">
+        <f>IF(OR(44&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M48" s="48">
+        <f>IF(OR(44&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11388,31 +11420,31 @@
           <t>n (ACTIVE)</t>
         </is>
       </c>
-      <c r="E49" s="47">
+      <c r="E49" s="50">
         <f>Analysis!G11</f>
         <v/>
       </c>
       <c r="H49" s="36" t="n">
         <v>45</v>
       </c>
-      <c r="I49" s="45">
-        <f>IF(Data!D49="""",NA(),Data!D49)</f>
-        <v/>
-      </c>
-      <c r="J49" s="45">
-        <f>IF(OR(Data!D49="""",Data!D48=""""),NA(),ABS(Data!D49-Data!D48))</f>
-        <v/>
-      </c>
-      <c r="K49" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L49" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M49" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I49" s="48">
+        <f>IF(OR(45&gt;$J$2,Data!D49=""),NA(),Data!D49)</f>
+        <v/>
+      </c>
+      <c r="J49" s="48">
+        <f>IF(OR(45&gt;$J$2,Data!D49="",Data!D48=""),NA(),ABS(Data!D49-Data!D48))</f>
+        <v/>
+      </c>
+      <c r="K49" s="48">
+        <f>IF(OR(45&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L49" s="48">
+        <f>IF(OR(45&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M49" s="48">
+        <f>IF(OR(45&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11438,24 +11470,24 @@
       <c r="H50" s="36" t="n">
         <v>46</v>
       </c>
-      <c r="I50" s="45">
-        <f>IF(Data!D50="""",NA(),Data!D50)</f>
-        <v/>
-      </c>
-      <c r="J50" s="45">
-        <f>IF(OR(Data!D50="""",Data!D49=""""),NA(),ABS(Data!D50-Data!D49))</f>
-        <v/>
-      </c>
-      <c r="K50" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L50" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M50" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I50" s="48">
+        <f>IF(OR(46&gt;$J$2,Data!D50=""),NA(),Data!D50)</f>
+        <v/>
+      </c>
+      <c r="J50" s="48">
+        <f>IF(OR(46&gt;$J$2,Data!D50="",Data!D49=""),NA(),ABS(Data!D50-Data!D49))</f>
+        <v/>
+      </c>
+      <c r="K50" s="48">
+        <f>IF(OR(46&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L50" s="48">
+        <f>IF(OR(46&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M50" s="48">
+        <f>IF(OR(46&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11463,24 +11495,24 @@
       <c r="H51" s="36" t="n">
         <v>47</v>
       </c>
-      <c r="I51" s="45">
-        <f>IF(Data!D51="""",NA(),Data!D51)</f>
-        <v/>
-      </c>
-      <c r="J51" s="45">
-        <f>IF(OR(Data!D51="""",Data!D50=""""),NA(),ABS(Data!D51-Data!D50))</f>
-        <v/>
-      </c>
-      <c r="K51" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L51" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M51" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I51" s="48">
+        <f>IF(OR(47&gt;$J$2,Data!D51=""),NA(),Data!D51)</f>
+        <v/>
+      </c>
+      <c r="J51" s="48">
+        <f>IF(OR(47&gt;$J$2,Data!D51="",Data!D50=""),NA(),ABS(Data!D51-Data!D50))</f>
+        <v/>
+      </c>
+      <c r="K51" s="48">
+        <f>IF(OR(47&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L51" s="48">
+        <f>IF(OR(47&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M51" s="48">
+        <f>IF(OR(47&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11488,24 +11520,24 @@
       <c r="H52" s="36" t="n">
         <v>48</v>
       </c>
-      <c r="I52" s="45">
-        <f>IF(Data!D52="""",NA(),Data!D52)</f>
-        <v/>
-      </c>
-      <c r="J52" s="45">
-        <f>IF(OR(Data!D52="""",Data!D51=""""),NA(),ABS(Data!D52-Data!D51))</f>
-        <v/>
-      </c>
-      <c r="K52" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L52" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M52" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I52" s="48">
+        <f>IF(OR(48&gt;$J$2,Data!D52=""),NA(),Data!D52)</f>
+        <v/>
+      </c>
+      <c r="J52" s="48">
+        <f>IF(OR(48&gt;$J$2,Data!D52="",Data!D51=""),NA(),ABS(Data!D52-Data!D51))</f>
+        <v/>
+      </c>
+      <c r="K52" s="48">
+        <f>IF(OR(48&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L52" s="48">
+        <f>IF(OR(48&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M52" s="48">
+        <f>IF(OR(48&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11513,24 +11545,24 @@
       <c r="H53" s="36" t="n">
         <v>49</v>
       </c>
-      <c r="I53" s="45">
-        <f>IF(Data!D53="""",NA(),Data!D53)</f>
-        <v/>
-      </c>
-      <c r="J53" s="45">
-        <f>IF(OR(Data!D53="""",Data!D52=""""),NA(),ABS(Data!D53-Data!D52))</f>
-        <v/>
-      </c>
-      <c r="K53" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L53" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M53" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I53" s="48">
+        <f>IF(OR(49&gt;$J$2,Data!D53=""),NA(),Data!D53)</f>
+        <v/>
+      </c>
+      <c r="J53" s="48">
+        <f>IF(OR(49&gt;$J$2,Data!D53="",Data!D52=""),NA(),ABS(Data!D53-Data!D52))</f>
+        <v/>
+      </c>
+      <c r="K53" s="48">
+        <f>IF(OR(49&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L53" s="48">
+        <f>IF(OR(49&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M53" s="48">
+        <f>IF(OR(49&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11538,24 +11570,1274 @@
       <c r="H54" s="36" t="n">
         <v>50</v>
       </c>
-      <c r="I54" s="45">
-        <f>IF(Data!D54="""",NA(),Data!D54)</f>
-        <v/>
-      </c>
-      <c r="J54" s="45">
-        <f>IF(OR(Data!D54="""",Data!D53=""""),NA(),ABS(Data!D54-Data!D53))</f>
-        <v/>
-      </c>
-      <c r="K54" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6,NA())</f>
-        <v/>
-      </c>
-      <c r="L54" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6+2.66*AVERAGE(J6:J54),NA())</f>
-        <v/>
-      </c>
-      <c r="M54" s="45">
-        <f>IF(Data!G5&gt;=2,Data!G6-2.66*AVERAGE(J6:J54),NA())</f>
+      <c r="I54" s="48">
+        <f>IF(OR(50&gt;$J$2,Data!D54=""),NA(),Data!D54)</f>
+        <v/>
+      </c>
+      <c r="J54" s="48">
+        <f>IF(OR(50&gt;$J$2,Data!D54="",Data!D53=""),NA(),ABS(Data!D54-Data!D53))</f>
+        <v/>
+      </c>
+      <c r="K54" s="48">
+        <f>IF(OR(50&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L54" s="48">
+        <f>IF(OR(50&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M54" s="48">
+        <f>IF(OR(50&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="H55" s="36" t="n">
+        <v>51</v>
+      </c>
+      <c r="I55" s="48">
+        <f>IF(OR(51&gt;$J$2,Data!D55=""),NA(),Data!D55)</f>
+        <v/>
+      </c>
+      <c r="J55" s="48">
+        <f>IF(OR(51&gt;$J$2,Data!D55="",Data!D54=""),NA(),ABS(Data!D55-Data!D54))</f>
+        <v/>
+      </c>
+      <c r="K55" s="48">
+        <f>IF(OR(51&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L55" s="48">
+        <f>IF(OR(51&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M55" s="48">
+        <f>IF(OR(51&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="H56" s="36" t="n">
+        <v>52</v>
+      </c>
+      <c r="I56" s="48">
+        <f>IF(OR(52&gt;$J$2,Data!D56=""),NA(),Data!D56)</f>
+        <v/>
+      </c>
+      <c r="J56" s="48">
+        <f>IF(OR(52&gt;$J$2,Data!D56="",Data!D55=""),NA(),ABS(Data!D56-Data!D55))</f>
+        <v/>
+      </c>
+      <c r="K56" s="48">
+        <f>IF(OR(52&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L56" s="48">
+        <f>IF(OR(52&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M56" s="48">
+        <f>IF(OR(52&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="H57" s="36" t="n">
+        <v>53</v>
+      </c>
+      <c r="I57" s="48">
+        <f>IF(OR(53&gt;$J$2,Data!D57=""),NA(),Data!D57)</f>
+        <v/>
+      </c>
+      <c r="J57" s="48">
+        <f>IF(OR(53&gt;$J$2,Data!D57="",Data!D56=""),NA(),ABS(Data!D57-Data!D56))</f>
+        <v/>
+      </c>
+      <c r="K57" s="48">
+        <f>IF(OR(53&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L57" s="48">
+        <f>IF(OR(53&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M57" s="48">
+        <f>IF(OR(53&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="H58" s="36" t="n">
+        <v>54</v>
+      </c>
+      <c r="I58" s="48">
+        <f>IF(OR(54&gt;$J$2,Data!D58=""),NA(),Data!D58)</f>
+        <v/>
+      </c>
+      <c r="J58" s="48">
+        <f>IF(OR(54&gt;$J$2,Data!D58="",Data!D57=""),NA(),ABS(Data!D58-Data!D57))</f>
+        <v/>
+      </c>
+      <c r="K58" s="48">
+        <f>IF(OR(54&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L58" s="48">
+        <f>IF(OR(54&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M58" s="48">
+        <f>IF(OR(54&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="H59" s="36" t="n">
+        <v>55</v>
+      </c>
+      <c r="I59" s="48">
+        <f>IF(OR(55&gt;$J$2,Data!D59=""),NA(),Data!D59)</f>
+        <v/>
+      </c>
+      <c r="J59" s="48">
+        <f>IF(OR(55&gt;$J$2,Data!D59="",Data!D58=""),NA(),ABS(Data!D59-Data!D58))</f>
+        <v/>
+      </c>
+      <c r="K59" s="48">
+        <f>IF(OR(55&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L59" s="48">
+        <f>IF(OR(55&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M59" s="48">
+        <f>IF(OR(55&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="H60" s="36" t="n">
+        <v>56</v>
+      </c>
+      <c r="I60" s="48">
+        <f>IF(OR(56&gt;$J$2,Data!D60=""),NA(),Data!D60)</f>
+        <v/>
+      </c>
+      <c r="J60" s="48">
+        <f>IF(OR(56&gt;$J$2,Data!D60="",Data!D59=""),NA(),ABS(Data!D60-Data!D59))</f>
+        <v/>
+      </c>
+      <c r="K60" s="48">
+        <f>IF(OR(56&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L60" s="48">
+        <f>IF(OR(56&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M60" s="48">
+        <f>IF(OR(56&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="H61" s="36" t="n">
+        <v>57</v>
+      </c>
+      <c r="I61" s="48">
+        <f>IF(OR(57&gt;$J$2,Data!D61=""),NA(),Data!D61)</f>
+        <v/>
+      </c>
+      <c r="J61" s="48">
+        <f>IF(OR(57&gt;$J$2,Data!D61="",Data!D60=""),NA(),ABS(Data!D61-Data!D60))</f>
+        <v/>
+      </c>
+      <c r="K61" s="48">
+        <f>IF(OR(57&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L61" s="48">
+        <f>IF(OR(57&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M61" s="48">
+        <f>IF(OR(57&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="H62" s="36" t="n">
+        <v>58</v>
+      </c>
+      <c r="I62" s="48">
+        <f>IF(OR(58&gt;$J$2,Data!D62=""),NA(),Data!D62)</f>
+        <v/>
+      </c>
+      <c r="J62" s="48">
+        <f>IF(OR(58&gt;$J$2,Data!D62="",Data!D61=""),NA(),ABS(Data!D62-Data!D61))</f>
+        <v/>
+      </c>
+      <c r="K62" s="48">
+        <f>IF(OR(58&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L62" s="48">
+        <f>IF(OR(58&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M62" s="48">
+        <f>IF(OR(58&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="H63" s="36" t="n">
+        <v>59</v>
+      </c>
+      <c r="I63" s="48">
+        <f>IF(OR(59&gt;$J$2,Data!D63=""),NA(),Data!D63)</f>
+        <v/>
+      </c>
+      <c r="J63" s="48">
+        <f>IF(OR(59&gt;$J$2,Data!D63="",Data!D62=""),NA(),ABS(Data!D63-Data!D62))</f>
+        <v/>
+      </c>
+      <c r="K63" s="48">
+        <f>IF(OR(59&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L63" s="48">
+        <f>IF(OR(59&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M63" s="48">
+        <f>IF(OR(59&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="H64" s="36" t="n">
+        <v>60</v>
+      </c>
+      <c r="I64" s="48">
+        <f>IF(OR(60&gt;$J$2,Data!D64=""),NA(),Data!D64)</f>
+        <v/>
+      </c>
+      <c r="J64" s="48">
+        <f>IF(OR(60&gt;$J$2,Data!D64="",Data!D63=""),NA(),ABS(Data!D64-Data!D63))</f>
+        <v/>
+      </c>
+      <c r="K64" s="48">
+        <f>IF(OR(60&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L64" s="48">
+        <f>IF(OR(60&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M64" s="48">
+        <f>IF(OR(60&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="H65" s="36" t="n">
+        <v>61</v>
+      </c>
+      <c r="I65" s="48">
+        <f>IF(OR(61&gt;$J$2,Data!D65=""),NA(),Data!D65)</f>
+        <v/>
+      </c>
+      <c r="J65" s="48">
+        <f>IF(OR(61&gt;$J$2,Data!D65="",Data!D64=""),NA(),ABS(Data!D65-Data!D64))</f>
+        <v/>
+      </c>
+      <c r="K65" s="48">
+        <f>IF(OR(61&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L65" s="48">
+        <f>IF(OR(61&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M65" s="48">
+        <f>IF(OR(61&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="H66" s="36" t="n">
+        <v>62</v>
+      </c>
+      <c r="I66" s="48">
+        <f>IF(OR(62&gt;$J$2,Data!D66=""),NA(),Data!D66)</f>
+        <v/>
+      </c>
+      <c r="J66" s="48">
+        <f>IF(OR(62&gt;$J$2,Data!D66="",Data!D65=""),NA(),ABS(Data!D66-Data!D65))</f>
+        <v/>
+      </c>
+      <c r="K66" s="48">
+        <f>IF(OR(62&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L66" s="48">
+        <f>IF(OR(62&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M66" s="48">
+        <f>IF(OR(62&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="H67" s="36" t="n">
+        <v>63</v>
+      </c>
+      <c r="I67" s="48">
+        <f>IF(OR(63&gt;$J$2,Data!D67=""),NA(),Data!D67)</f>
+        <v/>
+      </c>
+      <c r="J67" s="48">
+        <f>IF(OR(63&gt;$J$2,Data!D67="",Data!D66=""),NA(),ABS(Data!D67-Data!D66))</f>
+        <v/>
+      </c>
+      <c r="K67" s="48">
+        <f>IF(OR(63&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L67" s="48">
+        <f>IF(OR(63&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M67" s="48">
+        <f>IF(OR(63&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="H68" s="36" t="n">
+        <v>64</v>
+      </c>
+      <c r="I68" s="48">
+        <f>IF(OR(64&gt;$J$2,Data!D68=""),NA(),Data!D68)</f>
+        <v/>
+      </c>
+      <c r="J68" s="48">
+        <f>IF(OR(64&gt;$J$2,Data!D68="",Data!D67=""),NA(),ABS(Data!D68-Data!D67))</f>
+        <v/>
+      </c>
+      <c r="K68" s="48">
+        <f>IF(OR(64&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L68" s="48">
+        <f>IF(OR(64&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M68" s="48">
+        <f>IF(OR(64&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="H69" s="36" t="n">
+        <v>65</v>
+      </c>
+      <c r="I69" s="48">
+        <f>IF(OR(65&gt;$J$2,Data!D69=""),NA(),Data!D69)</f>
+        <v/>
+      </c>
+      <c r="J69" s="48">
+        <f>IF(OR(65&gt;$J$2,Data!D69="",Data!D68=""),NA(),ABS(Data!D69-Data!D68))</f>
+        <v/>
+      </c>
+      <c r="K69" s="48">
+        <f>IF(OR(65&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L69" s="48">
+        <f>IF(OR(65&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M69" s="48">
+        <f>IF(OR(65&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="H70" s="36" t="n">
+        <v>66</v>
+      </c>
+      <c r="I70" s="48">
+        <f>IF(OR(66&gt;$J$2,Data!D70=""),NA(),Data!D70)</f>
+        <v/>
+      </c>
+      <c r="J70" s="48">
+        <f>IF(OR(66&gt;$J$2,Data!D70="",Data!D69=""),NA(),ABS(Data!D70-Data!D69))</f>
+        <v/>
+      </c>
+      <c r="K70" s="48">
+        <f>IF(OR(66&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L70" s="48">
+        <f>IF(OR(66&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M70" s="48">
+        <f>IF(OR(66&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="H71" s="36" t="n">
+        <v>67</v>
+      </c>
+      <c r="I71" s="48">
+        <f>IF(OR(67&gt;$J$2,Data!D71=""),NA(),Data!D71)</f>
+        <v/>
+      </c>
+      <c r="J71" s="48">
+        <f>IF(OR(67&gt;$J$2,Data!D71="",Data!D70=""),NA(),ABS(Data!D71-Data!D70))</f>
+        <v/>
+      </c>
+      <c r="K71" s="48">
+        <f>IF(OR(67&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L71" s="48">
+        <f>IF(OR(67&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M71" s="48">
+        <f>IF(OR(67&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="H72" s="36" t="n">
+        <v>68</v>
+      </c>
+      <c r="I72" s="48">
+        <f>IF(OR(68&gt;$J$2,Data!D72=""),NA(),Data!D72)</f>
+        <v/>
+      </c>
+      <c r="J72" s="48">
+        <f>IF(OR(68&gt;$J$2,Data!D72="",Data!D71=""),NA(),ABS(Data!D72-Data!D71))</f>
+        <v/>
+      </c>
+      <c r="K72" s="48">
+        <f>IF(OR(68&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L72" s="48">
+        <f>IF(OR(68&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M72" s="48">
+        <f>IF(OR(68&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="H73" s="36" t="n">
+        <v>69</v>
+      </c>
+      <c r="I73" s="48">
+        <f>IF(OR(69&gt;$J$2,Data!D73=""),NA(),Data!D73)</f>
+        <v/>
+      </c>
+      <c r="J73" s="48">
+        <f>IF(OR(69&gt;$J$2,Data!D73="",Data!D72=""),NA(),ABS(Data!D73-Data!D72))</f>
+        <v/>
+      </c>
+      <c r="K73" s="48">
+        <f>IF(OR(69&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L73" s="48">
+        <f>IF(OR(69&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M73" s="48">
+        <f>IF(OR(69&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="H74" s="36" t="n">
+        <v>70</v>
+      </c>
+      <c r="I74" s="48">
+        <f>IF(OR(70&gt;$J$2,Data!D74=""),NA(),Data!D74)</f>
+        <v/>
+      </c>
+      <c r="J74" s="48">
+        <f>IF(OR(70&gt;$J$2,Data!D74="",Data!D73=""),NA(),ABS(Data!D74-Data!D73))</f>
+        <v/>
+      </c>
+      <c r="K74" s="48">
+        <f>IF(OR(70&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L74" s="48">
+        <f>IF(OR(70&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M74" s="48">
+        <f>IF(OR(70&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="H75" s="36" t="n">
+        <v>71</v>
+      </c>
+      <c r="I75" s="48">
+        <f>IF(OR(71&gt;$J$2,Data!D75=""),NA(),Data!D75)</f>
+        <v/>
+      </c>
+      <c r="J75" s="48">
+        <f>IF(OR(71&gt;$J$2,Data!D75="",Data!D74=""),NA(),ABS(Data!D75-Data!D74))</f>
+        <v/>
+      </c>
+      <c r="K75" s="48">
+        <f>IF(OR(71&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L75" s="48">
+        <f>IF(OR(71&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M75" s="48">
+        <f>IF(OR(71&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="H76" s="36" t="n">
+        <v>72</v>
+      </c>
+      <c r="I76" s="48">
+        <f>IF(OR(72&gt;$J$2,Data!D76=""),NA(),Data!D76)</f>
+        <v/>
+      </c>
+      <c r="J76" s="48">
+        <f>IF(OR(72&gt;$J$2,Data!D76="",Data!D75=""),NA(),ABS(Data!D76-Data!D75))</f>
+        <v/>
+      </c>
+      <c r="K76" s="48">
+        <f>IF(OR(72&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L76" s="48">
+        <f>IF(OR(72&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M76" s="48">
+        <f>IF(OR(72&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="H77" s="36" t="n">
+        <v>73</v>
+      </c>
+      <c r="I77" s="48">
+        <f>IF(OR(73&gt;$J$2,Data!D77=""),NA(),Data!D77)</f>
+        <v/>
+      </c>
+      <c r="J77" s="48">
+        <f>IF(OR(73&gt;$J$2,Data!D77="",Data!D76=""),NA(),ABS(Data!D77-Data!D76))</f>
+        <v/>
+      </c>
+      <c r="K77" s="48">
+        <f>IF(OR(73&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L77" s="48">
+        <f>IF(OR(73&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M77" s="48">
+        <f>IF(OR(73&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="H78" s="36" t="n">
+        <v>74</v>
+      </c>
+      <c r="I78" s="48">
+        <f>IF(OR(74&gt;$J$2,Data!D78=""),NA(),Data!D78)</f>
+        <v/>
+      </c>
+      <c r="J78" s="48">
+        <f>IF(OR(74&gt;$J$2,Data!D78="",Data!D77=""),NA(),ABS(Data!D78-Data!D77))</f>
+        <v/>
+      </c>
+      <c r="K78" s="48">
+        <f>IF(OR(74&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L78" s="48">
+        <f>IF(OR(74&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M78" s="48">
+        <f>IF(OR(74&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="H79" s="36" t="n">
+        <v>75</v>
+      </c>
+      <c r="I79" s="48">
+        <f>IF(OR(75&gt;$J$2,Data!D79=""),NA(),Data!D79)</f>
+        <v/>
+      </c>
+      <c r="J79" s="48">
+        <f>IF(OR(75&gt;$J$2,Data!D79="",Data!D78=""),NA(),ABS(Data!D79-Data!D78))</f>
+        <v/>
+      </c>
+      <c r="K79" s="48">
+        <f>IF(OR(75&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L79" s="48">
+        <f>IF(OR(75&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M79" s="48">
+        <f>IF(OR(75&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="H80" s="36" t="n">
+        <v>76</v>
+      </c>
+      <c r="I80" s="48">
+        <f>IF(OR(76&gt;$J$2,Data!D80=""),NA(),Data!D80)</f>
+        <v/>
+      </c>
+      <c r="J80" s="48">
+        <f>IF(OR(76&gt;$J$2,Data!D80="",Data!D79=""),NA(),ABS(Data!D80-Data!D79))</f>
+        <v/>
+      </c>
+      <c r="K80" s="48">
+        <f>IF(OR(76&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L80" s="48">
+        <f>IF(OR(76&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M80" s="48">
+        <f>IF(OR(76&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="H81" s="36" t="n">
+        <v>77</v>
+      </c>
+      <c r="I81" s="48">
+        <f>IF(OR(77&gt;$J$2,Data!D81=""),NA(),Data!D81)</f>
+        <v/>
+      </c>
+      <c r="J81" s="48">
+        <f>IF(OR(77&gt;$J$2,Data!D81="",Data!D80=""),NA(),ABS(Data!D81-Data!D80))</f>
+        <v/>
+      </c>
+      <c r="K81" s="48">
+        <f>IF(OR(77&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L81" s="48">
+        <f>IF(OR(77&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M81" s="48">
+        <f>IF(OR(77&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="H82" s="36" t="n">
+        <v>78</v>
+      </c>
+      <c r="I82" s="48">
+        <f>IF(OR(78&gt;$J$2,Data!D82=""),NA(),Data!D82)</f>
+        <v/>
+      </c>
+      <c r="J82" s="48">
+        <f>IF(OR(78&gt;$J$2,Data!D82="",Data!D81=""),NA(),ABS(Data!D82-Data!D81))</f>
+        <v/>
+      </c>
+      <c r="K82" s="48">
+        <f>IF(OR(78&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L82" s="48">
+        <f>IF(OR(78&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M82" s="48">
+        <f>IF(OR(78&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="H83" s="36" t="n">
+        <v>79</v>
+      </c>
+      <c r="I83" s="48">
+        <f>IF(OR(79&gt;$J$2,Data!D83=""),NA(),Data!D83)</f>
+        <v/>
+      </c>
+      <c r="J83" s="48">
+        <f>IF(OR(79&gt;$J$2,Data!D83="",Data!D82=""),NA(),ABS(Data!D83-Data!D82))</f>
+        <v/>
+      </c>
+      <c r="K83" s="48">
+        <f>IF(OR(79&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L83" s="48">
+        <f>IF(OR(79&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M83" s="48">
+        <f>IF(OR(79&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="H84" s="36" t="n">
+        <v>80</v>
+      </c>
+      <c r="I84" s="48">
+        <f>IF(OR(80&gt;$J$2,Data!D84=""),NA(),Data!D84)</f>
+        <v/>
+      </c>
+      <c r="J84" s="48">
+        <f>IF(OR(80&gt;$J$2,Data!D84="",Data!D83=""),NA(),ABS(Data!D84-Data!D83))</f>
+        <v/>
+      </c>
+      <c r="K84" s="48">
+        <f>IF(OR(80&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L84" s="48">
+        <f>IF(OR(80&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M84" s="48">
+        <f>IF(OR(80&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="H85" s="36" t="n">
+        <v>81</v>
+      </c>
+      <c r="I85" s="48">
+        <f>IF(OR(81&gt;$J$2,Data!D85=""),NA(),Data!D85)</f>
+        <v/>
+      </c>
+      <c r="J85" s="48">
+        <f>IF(OR(81&gt;$J$2,Data!D85="",Data!D84=""),NA(),ABS(Data!D85-Data!D84))</f>
+        <v/>
+      </c>
+      <c r="K85" s="48">
+        <f>IF(OR(81&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L85" s="48">
+        <f>IF(OR(81&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M85" s="48">
+        <f>IF(OR(81&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="H86" s="36" t="n">
+        <v>82</v>
+      </c>
+      <c r="I86" s="48">
+        <f>IF(OR(82&gt;$J$2,Data!D86=""),NA(),Data!D86)</f>
+        <v/>
+      </c>
+      <c r="J86" s="48">
+        <f>IF(OR(82&gt;$J$2,Data!D86="",Data!D85=""),NA(),ABS(Data!D86-Data!D85))</f>
+        <v/>
+      </c>
+      <c r="K86" s="48">
+        <f>IF(OR(82&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L86" s="48">
+        <f>IF(OR(82&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M86" s="48">
+        <f>IF(OR(82&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="H87" s="36" t="n">
+        <v>83</v>
+      </c>
+      <c r="I87" s="48">
+        <f>IF(OR(83&gt;$J$2,Data!D87=""),NA(),Data!D87)</f>
+        <v/>
+      </c>
+      <c r="J87" s="48">
+        <f>IF(OR(83&gt;$J$2,Data!D87="",Data!D86=""),NA(),ABS(Data!D87-Data!D86))</f>
+        <v/>
+      </c>
+      <c r="K87" s="48">
+        <f>IF(OR(83&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L87" s="48">
+        <f>IF(OR(83&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M87" s="48">
+        <f>IF(OR(83&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="H88" s="36" t="n">
+        <v>84</v>
+      </c>
+      <c r="I88" s="48">
+        <f>IF(OR(84&gt;$J$2,Data!D88=""),NA(),Data!D88)</f>
+        <v/>
+      </c>
+      <c r="J88" s="48">
+        <f>IF(OR(84&gt;$J$2,Data!D88="",Data!D87=""),NA(),ABS(Data!D88-Data!D87))</f>
+        <v/>
+      </c>
+      <c r="K88" s="48">
+        <f>IF(OR(84&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L88" s="48">
+        <f>IF(OR(84&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M88" s="48">
+        <f>IF(OR(84&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="H89" s="36" t="n">
+        <v>85</v>
+      </c>
+      <c r="I89" s="48">
+        <f>IF(OR(85&gt;$J$2,Data!D89=""),NA(),Data!D89)</f>
+        <v/>
+      </c>
+      <c r="J89" s="48">
+        <f>IF(OR(85&gt;$J$2,Data!D89="",Data!D88=""),NA(),ABS(Data!D89-Data!D88))</f>
+        <v/>
+      </c>
+      <c r="K89" s="48">
+        <f>IF(OR(85&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L89" s="48">
+        <f>IF(OR(85&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M89" s="48">
+        <f>IF(OR(85&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="H90" s="36" t="n">
+        <v>86</v>
+      </c>
+      <c r="I90" s="48">
+        <f>IF(OR(86&gt;$J$2,Data!D90=""),NA(),Data!D90)</f>
+        <v/>
+      </c>
+      <c r="J90" s="48">
+        <f>IF(OR(86&gt;$J$2,Data!D90="",Data!D89=""),NA(),ABS(Data!D90-Data!D89))</f>
+        <v/>
+      </c>
+      <c r="K90" s="48">
+        <f>IF(OR(86&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L90" s="48">
+        <f>IF(OR(86&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M90" s="48">
+        <f>IF(OR(86&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="H91" s="36" t="n">
+        <v>87</v>
+      </c>
+      <c r="I91" s="48">
+        <f>IF(OR(87&gt;$J$2,Data!D91=""),NA(),Data!D91)</f>
+        <v/>
+      </c>
+      <c r="J91" s="48">
+        <f>IF(OR(87&gt;$J$2,Data!D91="",Data!D90=""),NA(),ABS(Data!D91-Data!D90))</f>
+        <v/>
+      </c>
+      <c r="K91" s="48">
+        <f>IF(OR(87&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L91" s="48">
+        <f>IF(OR(87&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M91" s="48">
+        <f>IF(OR(87&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="H92" s="36" t="n">
+        <v>88</v>
+      </c>
+      <c r="I92" s="48">
+        <f>IF(OR(88&gt;$J$2,Data!D92=""),NA(),Data!D92)</f>
+        <v/>
+      </c>
+      <c r="J92" s="48">
+        <f>IF(OR(88&gt;$J$2,Data!D92="",Data!D91=""),NA(),ABS(Data!D92-Data!D91))</f>
+        <v/>
+      </c>
+      <c r="K92" s="48">
+        <f>IF(OR(88&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L92" s="48">
+        <f>IF(OR(88&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M92" s="48">
+        <f>IF(OR(88&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="H93" s="36" t="n">
+        <v>89</v>
+      </c>
+      <c r="I93" s="48">
+        <f>IF(OR(89&gt;$J$2,Data!D93=""),NA(),Data!D93)</f>
+        <v/>
+      </c>
+      <c r="J93" s="48">
+        <f>IF(OR(89&gt;$J$2,Data!D93="",Data!D92=""),NA(),ABS(Data!D93-Data!D92))</f>
+        <v/>
+      </c>
+      <c r="K93" s="48">
+        <f>IF(OR(89&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L93" s="48">
+        <f>IF(OR(89&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M93" s="48">
+        <f>IF(OR(89&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="H94" s="36" t="n">
+        <v>90</v>
+      </c>
+      <c r="I94" s="48">
+        <f>IF(OR(90&gt;$J$2,Data!D94=""),NA(),Data!D94)</f>
+        <v/>
+      </c>
+      <c r="J94" s="48">
+        <f>IF(OR(90&gt;$J$2,Data!D94="",Data!D93=""),NA(),ABS(Data!D94-Data!D93))</f>
+        <v/>
+      </c>
+      <c r="K94" s="48">
+        <f>IF(OR(90&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L94" s="48">
+        <f>IF(OR(90&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M94" s="48">
+        <f>IF(OR(90&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="H95" s="36" t="n">
+        <v>91</v>
+      </c>
+      <c r="I95" s="48">
+        <f>IF(OR(91&gt;$J$2,Data!D95=""),NA(),Data!D95)</f>
+        <v/>
+      </c>
+      <c r="J95" s="48">
+        <f>IF(OR(91&gt;$J$2,Data!D95="",Data!D94=""),NA(),ABS(Data!D95-Data!D94))</f>
+        <v/>
+      </c>
+      <c r="K95" s="48">
+        <f>IF(OR(91&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L95" s="48">
+        <f>IF(OR(91&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M95" s="48">
+        <f>IF(OR(91&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="H96" s="36" t="n">
+        <v>92</v>
+      </c>
+      <c r="I96" s="48">
+        <f>IF(OR(92&gt;$J$2,Data!D96=""),NA(),Data!D96)</f>
+        <v/>
+      </c>
+      <c r="J96" s="48">
+        <f>IF(OR(92&gt;$J$2,Data!D96="",Data!D95=""),NA(),ABS(Data!D96-Data!D95))</f>
+        <v/>
+      </c>
+      <c r="K96" s="48">
+        <f>IF(OR(92&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L96" s="48">
+        <f>IF(OR(92&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M96" s="48">
+        <f>IF(OR(92&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="H97" s="36" t="n">
+        <v>93</v>
+      </c>
+      <c r="I97" s="48">
+        <f>IF(OR(93&gt;$J$2,Data!D97=""),NA(),Data!D97)</f>
+        <v/>
+      </c>
+      <c r="J97" s="48">
+        <f>IF(OR(93&gt;$J$2,Data!D97="",Data!D96=""),NA(),ABS(Data!D97-Data!D96))</f>
+        <v/>
+      </c>
+      <c r="K97" s="48">
+        <f>IF(OR(93&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L97" s="48">
+        <f>IF(OR(93&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M97" s="48">
+        <f>IF(OR(93&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="H98" s="36" t="n">
+        <v>94</v>
+      </c>
+      <c r="I98" s="48">
+        <f>IF(OR(94&gt;$J$2,Data!D98=""),NA(),Data!D98)</f>
+        <v/>
+      </c>
+      <c r="J98" s="48">
+        <f>IF(OR(94&gt;$J$2,Data!D98="",Data!D97=""),NA(),ABS(Data!D98-Data!D97))</f>
+        <v/>
+      </c>
+      <c r="K98" s="48">
+        <f>IF(OR(94&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L98" s="48">
+        <f>IF(OR(94&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M98" s="48">
+        <f>IF(OR(94&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="H99" s="36" t="n">
+        <v>95</v>
+      </c>
+      <c r="I99" s="48">
+        <f>IF(OR(95&gt;$J$2,Data!D99=""),NA(),Data!D99)</f>
+        <v/>
+      </c>
+      <c r="J99" s="48">
+        <f>IF(OR(95&gt;$J$2,Data!D99="",Data!D98=""),NA(),ABS(Data!D99-Data!D98))</f>
+        <v/>
+      </c>
+      <c r="K99" s="48">
+        <f>IF(OR(95&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L99" s="48">
+        <f>IF(OR(95&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M99" s="48">
+        <f>IF(OR(95&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="H100" s="36" t="n">
+        <v>96</v>
+      </c>
+      <c r="I100" s="48">
+        <f>IF(OR(96&gt;$J$2,Data!D100=""),NA(),Data!D100)</f>
+        <v/>
+      </c>
+      <c r="J100" s="48">
+        <f>IF(OR(96&gt;$J$2,Data!D100="",Data!D99=""),NA(),ABS(Data!D100-Data!D99))</f>
+        <v/>
+      </c>
+      <c r="K100" s="48">
+        <f>IF(OR(96&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L100" s="48">
+        <f>IF(OR(96&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M100" s="48">
+        <f>IF(OR(96&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="H101" s="36" t="n">
+        <v>97</v>
+      </c>
+      <c r="I101" s="48">
+        <f>IF(OR(97&gt;$J$2,Data!D101=""),NA(),Data!D101)</f>
+        <v/>
+      </c>
+      <c r="J101" s="48">
+        <f>IF(OR(97&gt;$J$2,Data!D101="",Data!D100=""),NA(),ABS(Data!D101-Data!D100))</f>
+        <v/>
+      </c>
+      <c r="K101" s="48">
+        <f>IF(OR(97&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L101" s="48">
+        <f>IF(OR(97&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M101" s="48">
+        <f>IF(OR(97&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="H102" s="36" t="n">
+        <v>98</v>
+      </c>
+      <c r="I102" s="48">
+        <f>IF(OR(98&gt;$J$2,Data!D102=""),NA(),Data!D102)</f>
+        <v/>
+      </c>
+      <c r="J102" s="48">
+        <f>IF(OR(98&gt;$J$2,Data!D102="",Data!D101=""),NA(),ABS(Data!D102-Data!D101))</f>
+        <v/>
+      </c>
+      <c r="K102" s="48">
+        <f>IF(OR(98&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L102" s="48">
+        <f>IF(OR(98&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M102" s="48">
+        <f>IF(OR(98&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="H103" s="36" t="n">
+        <v>99</v>
+      </c>
+      <c r="I103" s="48">
+        <f>IF(OR(99&gt;$J$2,Data!D103=""),NA(),Data!D103)</f>
+        <v/>
+      </c>
+      <c r="J103" s="48">
+        <f>IF(OR(99&gt;$J$2,Data!D103="",Data!D102=""),NA(),ABS(Data!D103-Data!D102))</f>
+        <v/>
+      </c>
+      <c r="K103" s="48">
+        <f>IF(OR(99&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L103" s="48">
+        <f>IF(OR(99&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M103" s="48">
+        <f>IF(OR(99&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="H104" s="36" t="n">
+        <v>100</v>
+      </c>
+      <c r="I104" s="48">
+        <f>IF(OR(100&gt;$J$2,Data!D104=""),NA(),Data!D104)</f>
+        <v/>
+      </c>
+      <c r="J104" s="48">
+        <f>IF(OR(100&gt;$J$2,Data!D104="",Data!D103=""),NA(),ABS(Data!D104-Data!D103))</f>
+        <v/>
+      </c>
+      <c r="K104" s="48">
+        <f>IF(OR(100&gt;$J$2,Data!G5&lt;2),NA(),Data!G6)</f>
+        <v/>
+      </c>
+      <c r="L104" s="48">
+        <f>IF(OR(100&gt;$J$2,Data!G5&lt;2),NA(),Data!G6+2.66*AVERAGE(J6:J104))</f>
+        <v/>
+      </c>
+      <c r="M104" s="48">
+        <f>IF(OR(100&gt;$J$2,Data!G5&lt;2),NA(),Data!G6-2.66*AVERAGE(J6:J104))</f>
         <v/>
       </c>
     </row>
@@ -11567,6 +12849,11 @@
     <mergeCell ref="B46:E46"/>
     <mergeCell ref="H3:M3"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="I2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" promptTitle="Filter" prompt="Choose how many data points to show in control charts" type="list">
+      <formula1>"10,25,50,100,All"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -11686,59 +12973,59 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="48">
+      <c r="B4" s="51">
         <f>TODAY()</f>
         <v/>
       </c>
-      <c r="C4" s="49">
+      <c r="C4" s="52">
         <f>Analysis!C5</f>
         <v/>
       </c>
-      <c r="D4" s="49">
+      <c r="D4" s="52">
         <f>Analysis!C10</f>
         <v/>
       </c>
-      <c r="E4" s="50">
+      <c r="E4" s="53">
         <f>Analysis!C6</f>
         <v/>
       </c>
-      <c r="F4" s="50">
+      <c r="F4" s="53">
         <f>Analysis!C7</f>
         <v/>
       </c>
-      <c r="G4" s="50">
+      <c r="G4" s="53">
         <f>Analysis!C8</f>
         <v/>
       </c>
-      <c r="H4" s="51">
+      <c r="H4" s="54">
         <f>Analysis!G9</f>
         <v/>
       </c>
-      <c r="I4" s="51">
+      <c r="I4" s="54">
         <f>Analysis!G10</f>
         <v/>
       </c>
-      <c r="J4" s="52">
+      <c r="J4" s="55">
         <f>Analysis!G11</f>
         <v/>
       </c>
-      <c r="K4" s="50">
+      <c r="K4" s="53">
         <f>Analysis!G17</f>
         <v/>
       </c>
-      <c r="L4" s="50">
+      <c r="L4" s="53">
         <f>Analysis!G18</f>
         <v/>
       </c>
-      <c r="M4" s="53">
+      <c r="M4" s="56">
         <f>Analysis!J10</f>
         <v/>
       </c>
-      <c r="N4" s="50">
+      <c r="N4" s="53">
         <f>Analysis!G19</f>
         <v/>
       </c>
-      <c r="O4" s="49">
+      <c r="O4" s="52">
         <f>Analysis!B28</f>
         <v/>
       </c>
@@ -12591,325 +13878,325 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="54" t="inlineStr">
+      <c r="B1" s="57" t="inlineStr">
         <is>
           <t>Reference Guide — Formulas, Definitions &amp; How to Use</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="55" t="inlineStr"/>
+      <c r="B3" s="58" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="B4" s="56" t="inlineStr">
+      <c r="B4" s="59" t="inlineStr">
         <is>
           <t>How to Use This Workbook</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="55" t="inlineStr">
+      <c r="B5" s="58" t="inlineStr">
         <is>
           <t>1. Enter specifications (Tₘ, LSL, USL) in the Analysis sheet (blue cells)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="55" t="inlineStr">
+      <c r="B6" s="58" t="inlineStr">
         <is>
           <t>2. Choose Mode: 'Enter Manually' or 'Use Data Worksheet' (dropdown in C10)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="55" t="inlineStr">
+      <c r="B7" s="58" t="inlineStr">
         <is>
           <t>3. If Manual: enter x̄, σ, n directly in the Analysis sheet</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="55" t="inlineStr">
+      <c r="B8" s="58" t="inlineStr">
         <is>
           <t>4. If Worksheet: enter part data in the Data sheet — mean &amp; σ auto-link</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="55" t="inlineStr">
+      <c r="B9" s="58" t="inlineStr">
         <is>
           <t>5. All results, probability, hypothesis test, and verdict update INSTANTLY</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="55" t="inlineStr">
+      <c r="B10" s="58" t="inlineStr">
         <is>
           <t>6. View charts in the Charts sheet (bell curve + capability bars)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="55" t="inlineStr">
+      <c r="B11" s="58" t="inlineStr">
         <is>
           <t>7. To save a run: go to History sheet, copy Row 4, paste as VALUES into Row 5+</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="55" t="inlineStr"/>
+      <c r="B12" s="58" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="B13" s="56" t="inlineStr">
+      <c r="B13" s="59" t="inlineStr">
         <is>
           <t>Core Capability Formulas</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="55" t="inlineStr">
+      <c r="B14" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cp = (USL − LSL) / 6σ  — Potential capability if process is perfectly centered</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="55" t="inlineStr">
+      <c r="B15" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cpk = min[(USL − x̄) / 3σ,  (x̄ − LSL) / 3σ]  — Actual capability with centering error</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="55" t="inlineStr">
+      <c r="B16" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  Required Shift (Δ) = Tₘ − x̄  — How far to adjust the process mean</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="55" t="inlineStr">
+      <c r="B17" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  Required Tolerance = Target Index × 6σ  — Minimum tolerance band needed</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="55" t="inlineStr"/>
+      <c r="B18" s="58" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="B19" s="56" t="inlineStr">
+      <c r="B19" s="59" t="inlineStr">
         <is>
           <t>Capability Index Interpretation (Automotive Standards)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="55" t="inlineStr">
+      <c r="B20" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cpk ≥ 1.67  →  ✅ GOOD — Capable (standard automotive target)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="55" t="inlineStr">
+      <c r="B21" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.33 ≤ Cpk &lt; 1.67  →  ⚠ ACCEPTABLE — Meets minimum but below target</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="55" t="inlineStr">
+      <c r="B22" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.00 ≤ Cpk &lt; 1.33  →  ⚠ MARGINAL — High risk, improvement needed</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="55" t="inlineStr">
+      <c r="B23" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cpk &lt; 1.00  →  ❌ NOT CAPABLE — Produces significant defects</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="55" t="inlineStr"/>
+      <c r="B24" s="58" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="B25" s="56" t="inlineStr">
+      <c r="B25" s="59" t="inlineStr">
         <is>
           <t>Probability &amp; PPM</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="55" t="inlineStr">
+      <c r="B26" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  P(x &gt; USL) — Probability a part exceeds upper spec limit</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="55" t="inlineStr">
+      <c r="B27" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  P(x &lt; LSL) — Probability a part falls below lower spec limit</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="55" t="inlineStr">
+      <c r="B28" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  PPM = Probability × 1,000,000 — Parts Per Million defective</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="55" t="inlineStr"/>
+      <c r="B29" s="58" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="B30" s="56" t="inlineStr">
+      <c r="B30" s="59" t="inlineStr">
         <is>
           <t>Hypothesis Testing</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="55" t="inlineStr">
+      <c r="B31" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  H₀: μ = Tₘ (process is on target)</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="55" t="inlineStr">
+      <c r="B32" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  Z = (x̄ − Tₘ) / (σ / √n)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="55" t="inlineStr">
+      <c r="B33" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  p-value &lt; α → Reject H₀ → Significant shift detected</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="55" t="inlineStr">
+      <c r="B34" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  p-value ≥ α → Fail to Reject H₀ → No significant shift</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="55" t="inlineStr">
+      <c r="B35" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  Two-Sided: tests if mean differs in either direction</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="55" t="inlineStr">
+      <c r="B36" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  Upper-Sided: tests if mean is significantly above target</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="55" t="inlineStr">
+      <c r="B37" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  Lower-Sided: tests if mean is significantly below target</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="55" t="inlineStr"/>
+      <c r="B38" s="58" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="B39" s="56" t="inlineStr">
+      <c r="B39" s="59" t="inlineStr">
         <is>
           <t>Robustness Assessment</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="55" t="inlineStr">
+      <c r="B40" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  ROBUST: ±4σ spread contained within specification limits</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="55" t="inlineStr">
+      <c r="B41" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  MARGINAL: ±3σ contained but ±4σ is NOT — low tolerance for future shifts</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="55" t="inlineStr">
+      <c r="B42" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOT ROBUST: ±3σ breaches specification limits</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="55" t="inlineStr"/>
+      <c r="B43" s="58" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="B44" s="56" t="inlineStr">
+      <c r="B44" s="59" t="inlineStr">
         <is>
           <t>Spread Metrics</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="55" t="inlineStr">
+      <c r="B45" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  6σ Spread — Contains ~99.73% of process output (±3σ)</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="55" t="inlineStr">
+      <c r="B46" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  8σ Spread — Contains ~99.9937% of process output (±4σ)</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="55" t="inlineStr"/>
+      <c r="B47" s="58" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="B48" s="56" t="inlineStr">
+      <c r="B48" s="59" t="inlineStr">
         <is>
           <t>Color Coding</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="55" t="inlineStr">
+      <c r="B49" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  🟢 Green cells = Good / Capable / Within target</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="B50" s="55" t="inlineStr">
+      <c r="B50" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  🟡 Yellow cells = Warning / Marginal</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="B51" s="55" t="inlineStr">
+      <c r="B51" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔴 Red cells = Bad / Action Required / Not capable</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="B52" s="55" t="inlineStr">
+      <c r="B52" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔵 Blue cells = Input cells (enter your data here)</t>
         </is>

</xml_diff>

<commit_message>
Align Excel History & Reference sheets with Streamlit upgrades (tables, zones, standards)
</commit_message>
<xml_diff>
--- a/SPC_Statistical_Calculator.xlsx
+++ b/SPC_Statistical_Calculator.xlsx
@@ -32,7 +32,7 @@
     <numFmt numFmtId="170" formatCode=";;;"/>
     <numFmt numFmtId="171" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -143,6 +143,12 @@
     <font>
       <color rgb="00FFFFFF"/>
       <sz val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="9">
@@ -265,7 +271,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -404,12 +410,23 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -12866,24 +12883,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O54"/>
+  <dimension ref="B1:Q107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="36" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="36" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12913,60 +12932,70 @@
       </c>
       <c r="D3" s="35" t="inlineStr">
         <is>
+          <t>Characteristic</t>
+        </is>
+      </c>
+      <c r="E3" s="35" t="inlineStr">
+        <is>
           <t>Mode</t>
         </is>
       </c>
-      <c r="E3" s="35" t="inlineStr">
+      <c r="F3" s="35" t="inlineStr">
         <is>
           <t>Tₘ</t>
         </is>
       </c>
-      <c r="F3" s="35" t="inlineStr">
+      <c r="G3" s="35" t="inlineStr">
         <is>
           <t>LSL</t>
         </is>
       </c>
-      <c r="G3" s="35" t="inlineStr">
+      <c r="H3" s="35" t="inlineStr">
         <is>
           <t>USL</t>
         </is>
       </c>
-      <c r="H3" s="35" t="inlineStr">
+      <c r="I3" s="35" t="inlineStr">
         <is>
           <t>x̄</t>
         </is>
       </c>
-      <c r="I3" s="35" t="inlineStr">
+      <c r="J3" s="35" t="inlineStr">
         <is>
           <t>σ</t>
         </is>
       </c>
-      <c r="J3" s="35" t="inlineStr">
+      <c r="K3" s="35" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="K3" s="35" t="inlineStr">
+      <c r="L3" s="35" t="inlineStr">
         <is>
           <t>Cp</t>
         </is>
       </c>
-      <c r="L3" s="35" t="inlineStr">
+      <c r="M3" s="35" t="inlineStr">
         <is>
           <t>Cpk</t>
         </is>
       </c>
-      <c r="M3" s="35" t="inlineStr">
-        <is>
-          <t>PPM Total</t>
-        </is>
-      </c>
       <c r="N3" s="35" t="inlineStr">
         <is>
           <t>Shift (Δ)</t>
         </is>
       </c>
       <c r="O3" s="35" t="inlineStr">
+        <is>
+          <t>PPM &lt; LSL</t>
+        </is>
+      </c>
+      <c r="P3" s="35" t="inlineStr">
+        <is>
+          <t>PPM &gt; USL</t>
+        </is>
+      </c>
+      <c r="Q3" s="35" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
@@ -12982,50 +13011,58 @@
         <v/>
       </c>
       <c r="D4" s="52">
+        <f>Analysis!C4</f>
+        <v/>
+      </c>
+      <c r="E4" s="52">
         <f>Analysis!C10</f>
         <v/>
       </c>
-      <c r="E4" s="53">
+      <c r="F4" s="53">
         <f>Analysis!C6</f>
         <v/>
       </c>
-      <c r="F4" s="53">
+      <c r="G4" s="53">
         <f>Analysis!C7</f>
         <v/>
       </c>
-      <c r="G4" s="53">
+      <c r="H4" s="53">
         <f>Analysis!C8</f>
         <v/>
       </c>
-      <c r="H4" s="54">
+      <c r="I4" s="54">
         <f>Analysis!G9</f>
         <v/>
       </c>
-      <c r="I4" s="54">
+      <c r="J4" s="54">
         <f>Analysis!G10</f>
         <v/>
       </c>
-      <c r="J4" s="55">
+      <c r="K4" s="55">
         <f>Analysis!G11</f>
         <v/>
       </c>
-      <c r="K4" s="53">
+      <c r="L4" s="53">
         <f>Analysis!G17</f>
         <v/>
       </c>
-      <c r="L4" s="53">
+      <c r="M4" s="53">
         <f>Analysis!G18</f>
-        <v/>
-      </c>
-      <c r="M4" s="56">
-        <f>Analysis!J10</f>
         <v/>
       </c>
       <c r="N4" s="53">
         <f>Analysis!G19</f>
         <v/>
       </c>
-      <c r="O4" s="52">
+      <c r="O4" s="56">
+        <f>Analysis!I9</f>
+        <v/>
+      </c>
+      <c r="P4" s="56">
+        <f>Analysis!I10</f>
+        <v/>
+      </c>
+      <c r="Q4" s="52">
         <f>Analysis!B28</f>
         <v/>
       </c>
@@ -13045,6 +13082,8 @@
       <c r="M5" s="39" t="n"/>
       <c r="N5" s="39" t="n"/>
       <c r="O5" s="39" t="n"/>
+      <c r="P5" s="39" t="n"/>
+      <c r="Q5" s="39" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="37" t="n"/>
@@ -13061,6 +13100,8 @@
       <c r="M6" s="37" t="n"/>
       <c r="N6" s="37" t="n"/>
       <c r="O6" s="37" t="n"/>
+      <c r="P6" s="37" t="n"/>
+      <c r="Q6" s="37" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="39" t="n"/>
@@ -13077,6 +13118,8 @@
       <c r="M7" s="39" t="n"/>
       <c r="N7" s="39" t="n"/>
       <c r="O7" s="39" t="n"/>
+      <c r="P7" s="39" t="n"/>
+      <c r="Q7" s="39" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="37" t="n"/>
@@ -13093,6 +13136,8 @@
       <c r="M8" s="37" t="n"/>
       <c r="N8" s="37" t="n"/>
       <c r="O8" s="37" t="n"/>
+      <c r="P8" s="37" t="n"/>
+      <c r="Q8" s="37" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="39" t="n"/>
@@ -13109,6 +13154,8 @@
       <c r="M9" s="39" t="n"/>
       <c r="N9" s="39" t="n"/>
       <c r="O9" s="39" t="n"/>
+      <c r="P9" s="39" t="n"/>
+      <c r="Q9" s="39" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="37" t="n"/>
@@ -13125,6 +13172,8 @@
       <c r="M10" s="37" t="n"/>
       <c r="N10" s="37" t="n"/>
       <c r="O10" s="37" t="n"/>
+      <c r="P10" s="37" t="n"/>
+      <c r="Q10" s="37" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="39" t="n"/>
@@ -13141,6 +13190,8 @@
       <c r="M11" s="39" t="n"/>
       <c r="N11" s="39" t="n"/>
       <c r="O11" s="39" t="n"/>
+      <c r="P11" s="39" t="n"/>
+      <c r="Q11" s="39" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="37" t="n"/>
@@ -13157,6 +13208,8 @@
       <c r="M12" s="37" t="n"/>
       <c r="N12" s="37" t="n"/>
       <c r="O12" s="37" t="n"/>
+      <c r="P12" s="37" t="n"/>
+      <c r="Q12" s="37" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="39" t="n"/>
@@ -13173,6 +13226,8 @@
       <c r="M13" s="39" t="n"/>
       <c r="N13" s="39" t="n"/>
       <c r="O13" s="39" t="n"/>
+      <c r="P13" s="39" t="n"/>
+      <c r="Q13" s="39" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="37" t="n"/>
@@ -13189,6 +13244,8 @@
       <c r="M14" s="37" t="n"/>
       <c r="N14" s="37" t="n"/>
       <c r="O14" s="37" t="n"/>
+      <c r="P14" s="37" t="n"/>
+      <c r="Q14" s="37" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="39" t="n"/>
@@ -13205,6 +13262,8 @@
       <c r="M15" s="39" t="n"/>
       <c r="N15" s="39" t="n"/>
       <c r="O15" s="39" t="n"/>
+      <c r="P15" s="39" t="n"/>
+      <c r="Q15" s="39" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="37" t="n"/>
@@ -13221,6 +13280,8 @@
       <c r="M16" s="37" t="n"/>
       <c r="N16" s="37" t="n"/>
       <c r="O16" s="37" t="n"/>
+      <c r="P16" s="37" t="n"/>
+      <c r="Q16" s="37" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="39" t="n"/>
@@ -13237,6 +13298,8 @@
       <c r="M17" s="39" t="n"/>
       <c r="N17" s="39" t="n"/>
       <c r="O17" s="39" t="n"/>
+      <c r="P17" s="39" t="n"/>
+      <c r="Q17" s="39" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="37" t="n"/>
@@ -13253,6 +13316,8 @@
       <c r="M18" s="37" t="n"/>
       <c r="N18" s="37" t="n"/>
       <c r="O18" s="37" t="n"/>
+      <c r="P18" s="37" t="n"/>
+      <c r="Q18" s="37" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="39" t="n"/>
@@ -13269,6 +13334,8 @@
       <c r="M19" s="39" t="n"/>
       <c r="N19" s="39" t="n"/>
       <c r="O19" s="39" t="n"/>
+      <c r="P19" s="39" t="n"/>
+      <c r="Q19" s="39" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="37" t="n"/>
@@ -13285,6 +13352,8 @@
       <c r="M20" s="37" t="n"/>
       <c r="N20" s="37" t="n"/>
       <c r="O20" s="37" t="n"/>
+      <c r="P20" s="37" t="n"/>
+      <c r="Q20" s="37" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="39" t="n"/>
@@ -13301,6 +13370,8 @@
       <c r="M21" s="39" t="n"/>
       <c r="N21" s="39" t="n"/>
       <c r="O21" s="39" t="n"/>
+      <c r="P21" s="39" t="n"/>
+      <c r="Q21" s="39" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="37" t="n"/>
@@ -13317,6 +13388,8 @@
       <c r="M22" s="37" t="n"/>
       <c r="N22" s="37" t="n"/>
       <c r="O22" s="37" t="n"/>
+      <c r="P22" s="37" t="n"/>
+      <c r="Q22" s="37" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="39" t="n"/>
@@ -13333,6 +13406,8 @@
       <c r="M23" s="39" t="n"/>
       <c r="N23" s="39" t="n"/>
       <c r="O23" s="39" t="n"/>
+      <c r="P23" s="39" t="n"/>
+      <c r="Q23" s="39" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="37" t="n"/>
@@ -13349,6 +13424,8 @@
       <c r="M24" s="37" t="n"/>
       <c r="N24" s="37" t="n"/>
       <c r="O24" s="37" t="n"/>
+      <c r="P24" s="37" t="n"/>
+      <c r="Q24" s="37" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="39" t="n"/>
@@ -13365,6 +13442,8 @@
       <c r="M25" s="39" t="n"/>
       <c r="N25" s="39" t="n"/>
       <c r="O25" s="39" t="n"/>
+      <c r="P25" s="39" t="n"/>
+      <c r="Q25" s="39" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="37" t="n"/>
@@ -13381,6 +13460,8 @@
       <c r="M26" s="37" t="n"/>
       <c r="N26" s="37" t="n"/>
       <c r="O26" s="37" t="n"/>
+      <c r="P26" s="37" t="n"/>
+      <c r="Q26" s="37" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="39" t="n"/>
@@ -13397,6 +13478,8 @@
       <c r="M27" s="39" t="n"/>
       <c r="N27" s="39" t="n"/>
       <c r="O27" s="39" t="n"/>
+      <c r="P27" s="39" t="n"/>
+      <c r="Q27" s="39" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="37" t="n"/>
@@ -13413,6 +13496,8 @@
       <c r="M28" s="37" t="n"/>
       <c r="N28" s="37" t="n"/>
       <c r="O28" s="37" t="n"/>
+      <c r="P28" s="37" t="n"/>
+      <c r="Q28" s="37" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="39" t="n"/>
@@ -13429,6 +13514,8 @@
       <c r="M29" s="39" t="n"/>
       <c r="N29" s="39" t="n"/>
       <c r="O29" s="39" t="n"/>
+      <c r="P29" s="39" t="n"/>
+      <c r="Q29" s="39" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="37" t="n"/>
@@ -13445,6 +13532,8 @@
       <c r="M30" s="37" t="n"/>
       <c r="N30" s="37" t="n"/>
       <c r="O30" s="37" t="n"/>
+      <c r="P30" s="37" t="n"/>
+      <c r="Q30" s="37" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="39" t="n"/>
@@ -13461,6 +13550,8 @@
       <c r="M31" s="39" t="n"/>
       <c r="N31" s="39" t="n"/>
       <c r="O31" s="39" t="n"/>
+      <c r="P31" s="39" t="n"/>
+      <c r="Q31" s="39" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="37" t="n"/>
@@ -13477,6 +13568,8 @@
       <c r="M32" s="37" t="n"/>
       <c r="N32" s="37" t="n"/>
       <c r="O32" s="37" t="n"/>
+      <c r="P32" s="37" t="n"/>
+      <c r="Q32" s="37" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="39" t="n"/>
@@ -13493,6 +13586,8 @@
       <c r="M33" s="39" t="n"/>
       <c r="N33" s="39" t="n"/>
       <c r="O33" s="39" t="n"/>
+      <c r="P33" s="39" t="n"/>
+      <c r="Q33" s="39" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="37" t="n"/>
@@ -13509,6 +13604,8 @@
       <c r="M34" s="37" t="n"/>
       <c r="N34" s="37" t="n"/>
       <c r="O34" s="37" t="n"/>
+      <c r="P34" s="37" t="n"/>
+      <c r="Q34" s="37" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="39" t="n"/>
@@ -13525,6 +13622,8 @@
       <c r="M35" s="39" t="n"/>
       <c r="N35" s="39" t="n"/>
       <c r="O35" s="39" t="n"/>
+      <c r="P35" s="39" t="n"/>
+      <c r="Q35" s="39" t="n"/>
     </row>
     <row r="36">
       <c r="B36" s="37" t="n"/>
@@ -13541,6 +13640,8 @@
       <c r="M36" s="37" t="n"/>
       <c r="N36" s="37" t="n"/>
       <c r="O36" s="37" t="n"/>
+      <c r="P36" s="37" t="n"/>
+      <c r="Q36" s="37" t="n"/>
     </row>
     <row r="37">
       <c r="B37" s="39" t="n"/>
@@ -13557,6 +13658,8 @@
       <c r="M37" s="39" t="n"/>
       <c r="N37" s="39" t="n"/>
       <c r="O37" s="39" t="n"/>
+      <c r="P37" s="39" t="n"/>
+      <c r="Q37" s="39" t="n"/>
     </row>
     <row r="38">
       <c r="B38" s="37" t="n"/>
@@ -13573,6 +13676,8 @@
       <c r="M38" s="37" t="n"/>
       <c r="N38" s="37" t="n"/>
       <c r="O38" s="37" t="n"/>
+      <c r="P38" s="37" t="n"/>
+      <c r="Q38" s="37" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="39" t="n"/>
@@ -13589,6 +13694,8 @@
       <c r="M39" s="39" t="n"/>
       <c r="N39" s="39" t="n"/>
       <c r="O39" s="39" t="n"/>
+      <c r="P39" s="39" t="n"/>
+      <c r="Q39" s="39" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="37" t="n"/>
@@ -13605,6 +13712,8 @@
       <c r="M40" s="37" t="n"/>
       <c r="N40" s="37" t="n"/>
       <c r="O40" s="37" t="n"/>
+      <c r="P40" s="37" t="n"/>
+      <c r="Q40" s="37" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="39" t="n"/>
@@ -13621,6 +13730,8 @@
       <c r="M41" s="39" t="n"/>
       <c r="N41" s="39" t="n"/>
       <c r="O41" s="39" t="n"/>
+      <c r="P41" s="39" t="n"/>
+      <c r="Q41" s="39" t="n"/>
     </row>
     <row r="42">
       <c r="B42" s="37" t="n"/>
@@ -13637,6 +13748,8 @@
       <c r="M42" s="37" t="n"/>
       <c r="N42" s="37" t="n"/>
       <c r="O42" s="37" t="n"/>
+      <c r="P42" s="37" t="n"/>
+      <c r="Q42" s="37" t="n"/>
     </row>
     <row r="43">
       <c r="B43" s="39" t="n"/>
@@ -13653,6 +13766,8 @@
       <c r="M43" s="39" t="n"/>
       <c r="N43" s="39" t="n"/>
       <c r="O43" s="39" t="n"/>
+      <c r="P43" s="39" t="n"/>
+      <c r="Q43" s="39" t="n"/>
     </row>
     <row r="44">
       <c r="B44" s="37" t="n"/>
@@ -13669,6 +13784,8 @@
       <c r="M44" s="37" t="n"/>
       <c r="N44" s="37" t="n"/>
       <c r="O44" s="37" t="n"/>
+      <c r="P44" s="37" t="n"/>
+      <c r="Q44" s="37" t="n"/>
     </row>
     <row r="45">
       <c r="B45" s="39" t="n"/>
@@ -13685,6 +13802,8 @@
       <c r="M45" s="39" t="n"/>
       <c r="N45" s="39" t="n"/>
       <c r="O45" s="39" t="n"/>
+      <c r="P45" s="39" t="n"/>
+      <c r="Q45" s="39" t="n"/>
     </row>
     <row r="46">
       <c r="B46" s="37" t="n"/>
@@ -13701,6 +13820,8 @@
       <c r="M46" s="37" t="n"/>
       <c r="N46" s="37" t="n"/>
       <c r="O46" s="37" t="n"/>
+      <c r="P46" s="37" t="n"/>
+      <c r="Q46" s="37" t="n"/>
     </row>
     <row r="47">
       <c r="B47" s="39" t="n"/>
@@ -13717,6 +13838,8 @@
       <c r="M47" s="39" t="n"/>
       <c r="N47" s="39" t="n"/>
       <c r="O47" s="39" t="n"/>
+      <c r="P47" s="39" t="n"/>
+      <c r="Q47" s="39" t="n"/>
     </row>
     <row r="48">
       <c r="B48" s="37" t="n"/>
@@ -13733,6 +13856,8 @@
       <c r="M48" s="37" t="n"/>
       <c r="N48" s="37" t="n"/>
       <c r="O48" s="37" t="n"/>
+      <c r="P48" s="37" t="n"/>
+      <c r="Q48" s="37" t="n"/>
     </row>
     <row r="49">
       <c r="B49" s="39" t="n"/>
@@ -13749,6 +13874,8 @@
       <c r="M49" s="39" t="n"/>
       <c r="N49" s="39" t="n"/>
       <c r="O49" s="39" t="n"/>
+      <c r="P49" s="39" t="n"/>
+      <c r="Q49" s="39" t="n"/>
     </row>
     <row r="50">
       <c r="B50" s="37" t="n"/>
@@ -13765,6 +13892,8 @@
       <c r="M50" s="37" t="n"/>
       <c r="N50" s="37" t="n"/>
       <c r="O50" s="37" t="n"/>
+      <c r="P50" s="37" t="n"/>
+      <c r="Q50" s="37" t="n"/>
     </row>
     <row r="51">
       <c r="B51" s="39" t="n"/>
@@ -13781,6 +13910,8 @@
       <c r="M51" s="39" t="n"/>
       <c r="N51" s="39" t="n"/>
       <c r="O51" s="39" t="n"/>
+      <c r="P51" s="39" t="n"/>
+      <c r="Q51" s="39" t="n"/>
     </row>
     <row r="52">
       <c r="B52" s="37" t="n"/>
@@ -13797,6 +13928,8 @@
       <c r="M52" s="37" t="n"/>
       <c r="N52" s="37" t="n"/>
       <c r="O52" s="37" t="n"/>
+      <c r="P52" s="37" t="n"/>
+      <c r="Q52" s="37" t="n"/>
     </row>
     <row r="53">
       <c r="B53" s="39" t="n"/>
@@ -13813,6 +13946,8 @@
       <c r="M53" s="39" t="n"/>
       <c r="N53" s="39" t="n"/>
       <c r="O53" s="39" t="n"/>
+      <c r="P53" s="39" t="n"/>
+      <c r="Q53" s="39" t="n"/>
     </row>
     <row r="54">
       <c r="B54" s="37" t="n"/>
@@ -13829,13 +13964,923 @@
       <c r="M54" s="37" t="n"/>
       <c r="N54" s="37" t="n"/>
       <c r="O54" s="37" t="n"/>
+      <c r="P54" s="37" t="n"/>
+      <c r="Q54" s="37" t="n"/>
+    </row>
+    <row r="55">
+      <c r="B55" s="39" t="n"/>
+      <c r="C55" s="39" t="n"/>
+      <c r="D55" s="39" t="n"/>
+      <c r="E55" s="39" t="n"/>
+      <c r="F55" s="39" t="n"/>
+      <c r="G55" s="39" t="n"/>
+      <c r="H55" s="39" t="n"/>
+      <c r="I55" s="39" t="n"/>
+      <c r="J55" s="39" t="n"/>
+      <c r="K55" s="39" t="n"/>
+      <c r="L55" s="39" t="n"/>
+      <c r="M55" s="39" t="n"/>
+      <c r="N55" s="39" t="n"/>
+      <c r="O55" s="39" t="n"/>
+      <c r="P55" s="39" t="n"/>
+      <c r="Q55" s="39" t="n"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="37" t="n"/>
+      <c r="C56" s="37" t="n"/>
+      <c r="D56" s="37" t="n"/>
+      <c r="E56" s="37" t="n"/>
+      <c r="F56" s="37" t="n"/>
+      <c r="G56" s="37" t="n"/>
+      <c r="H56" s="37" t="n"/>
+      <c r="I56" s="37" t="n"/>
+      <c r="J56" s="37" t="n"/>
+      <c r="K56" s="37" t="n"/>
+      <c r="L56" s="37" t="n"/>
+      <c r="M56" s="37" t="n"/>
+      <c r="N56" s="37" t="n"/>
+      <c r="O56" s="37" t="n"/>
+      <c r="P56" s="37" t="n"/>
+      <c r="Q56" s="37" t="n"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="39" t="n"/>
+      <c r="C57" s="39" t="n"/>
+      <c r="D57" s="39" t="n"/>
+      <c r="E57" s="39" t="n"/>
+      <c r="F57" s="39" t="n"/>
+      <c r="G57" s="39" t="n"/>
+      <c r="H57" s="39" t="n"/>
+      <c r="I57" s="39" t="n"/>
+      <c r="J57" s="39" t="n"/>
+      <c r="K57" s="39" t="n"/>
+      <c r="L57" s="39" t="n"/>
+      <c r="M57" s="39" t="n"/>
+      <c r="N57" s="39" t="n"/>
+      <c r="O57" s="39" t="n"/>
+      <c r="P57" s="39" t="n"/>
+      <c r="Q57" s="39" t="n"/>
+    </row>
+    <row r="58">
+      <c r="B58" s="37" t="n"/>
+      <c r="C58" s="37" t="n"/>
+      <c r="D58" s="37" t="n"/>
+      <c r="E58" s="37" t="n"/>
+      <c r="F58" s="37" t="n"/>
+      <c r="G58" s="37" t="n"/>
+      <c r="H58" s="37" t="n"/>
+      <c r="I58" s="37" t="n"/>
+      <c r="J58" s="37" t="n"/>
+      <c r="K58" s="37" t="n"/>
+      <c r="L58" s="37" t="n"/>
+      <c r="M58" s="37" t="n"/>
+      <c r="N58" s="37" t="n"/>
+      <c r="O58" s="37" t="n"/>
+      <c r="P58" s="37" t="n"/>
+      <c r="Q58" s="37" t="n"/>
+    </row>
+    <row r="59">
+      <c r="B59" s="39" t="n"/>
+      <c r="C59" s="39" t="n"/>
+      <c r="D59" s="39" t="n"/>
+      <c r="E59" s="39" t="n"/>
+      <c r="F59" s="39" t="n"/>
+      <c r="G59" s="39" t="n"/>
+      <c r="H59" s="39" t="n"/>
+      <c r="I59" s="39" t="n"/>
+      <c r="J59" s="39" t="n"/>
+      <c r="K59" s="39" t="n"/>
+      <c r="L59" s="39" t="n"/>
+      <c r="M59" s="39" t="n"/>
+      <c r="N59" s="39" t="n"/>
+      <c r="O59" s="39" t="n"/>
+      <c r="P59" s="39" t="n"/>
+      <c r="Q59" s="39" t="n"/>
+    </row>
+    <row r="60">
+      <c r="B60" s="37" t="n"/>
+      <c r="C60" s="37" t="n"/>
+      <c r="D60" s="37" t="n"/>
+      <c r="E60" s="37" t="n"/>
+      <c r="F60" s="37" t="n"/>
+      <c r="G60" s="37" t="n"/>
+      <c r="H60" s="37" t="n"/>
+      <c r="I60" s="37" t="n"/>
+      <c r="J60" s="37" t="n"/>
+      <c r="K60" s="37" t="n"/>
+      <c r="L60" s="37" t="n"/>
+      <c r="M60" s="37" t="n"/>
+      <c r="N60" s="37" t="n"/>
+      <c r="O60" s="37" t="n"/>
+      <c r="P60" s="37" t="n"/>
+      <c r="Q60" s="37" t="n"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="39" t="n"/>
+      <c r="C61" s="39" t="n"/>
+      <c r="D61" s="39" t="n"/>
+      <c r="E61" s="39" t="n"/>
+      <c r="F61" s="39" t="n"/>
+      <c r="G61" s="39" t="n"/>
+      <c r="H61" s="39" t="n"/>
+      <c r="I61" s="39" t="n"/>
+      <c r="J61" s="39" t="n"/>
+      <c r="K61" s="39" t="n"/>
+      <c r="L61" s="39" t="n"/>
+      <c r="M61" s="39" t="n"/>
+      <c r="N61" s="39" t="n"/>
+      <c r="O61" s="39" t="n"/>
+      <c r="P61" s="39" t="n"/>
+      <c r="Q61" s="39" t="n"/>
+    </row>
+    <row r="62">
+      <c r="B62" s="37" t="n"/>
+      <c r="C62" s="37" t="n"/>
+      <c r="D62" s="37" t="n"/>
+      <c r="E62" s="37" t="n"/>
+      <c r="F62" s="37" t="n"/>
+      <c r="G62" s="37" t="n"/>
+      <c r="H62" s="37" t="n"/>
+      <c r="I62" s="37" t="n"/>
+      <c r="J62" s="37" t="n"/>
+      <c r="K62" s="37" t="n"/>
+      <c r="L62" s="37" t="n"/>
+      <c r="M62" s="37" t="n"/>
+      <c r="N62" s="37" t="n"/>
+      <c r="O62" s="37" t="n"/>
+      <c r="P62" s="37" t="n"/>
+      <c r="Q62" s="37" t="n"/>
+    </row>
+    <row r="63">
+      <c r="B63" s="39" t="n"/>
+      <c r="C63" s="39" t="n"/>
+      <c r="D63" s="39" t="n"/>
+      <c r="E63" s="39" t="n"/>
+      <c r="F63" s="39" t="n"/>
+      <c r="G63" s="39" t="n"/>
+      <c r="H63" s="39" t="n"/>
+      <c r="I63" s="39" t="n"/>
+      <c r="J63" s="39" t="n"/>
+      <c r="K63" s="39" t="n"/>
+      <c r="L63" s="39" t="n"/>
+      <c r="M63" s="39" t="n"/>
+      <c r="N63" s="39" t="n"/>
+      <c r="O63" s="39" t="n"/>
+      <c r="P63" s="39" t="n"/>
+      <c r="Q63" s="39" t="n"/>
+    </row>
+    <row r="64">
+      <c r="B64" s="37" t="n"/>
+      <c r="C64" s="37" t="n"/>
+      <c r="D64" s="37" t="n"/>
+      <c r="E64" s="37" t="n"/>
+      <c r="F64" s="37" t="n"/>
+      <c r="G64" s="37" t="n"/>
+      <c r="H64" s="37" t="n"/>
+      <c r="I64" s="37" t="n"/>
+      <c r="J64" s="37" t="n"/>
+      <c r="K64" s="37" t="n"/>
+      <c r="L64" s="37" t="n"/>
+      <c r="M64" s="37" t="n"/>
+      <c r="N64" s="37" t="n"/>
+      <c r="O64" s="37" t="n"/>
+      <c r="P64" s="37" t="n"/>
+      <c r="Q64" s="37" t="n"/>
+    </row>
+    <row r="65">
+      <c r="B65" s="39" t="n"/>
+      <c r="C65" s="39" t="n"/>
+      <c r="D65" s="39" t="n"/>
+      <c r="E65" s="39" t="n"/>
+      <c r="F65" s="39" t="n"/>
+      <c r="G65" s="39" t="n"/>
+      <c r="H65" s="39" t="n"/>
+      <c r="I65" s="39" t="n"/>
+      <c r="J65" s="39" t="n"/>
+      <c r="K65" s="39" t="n"/>
+      <c r="L65" s="39" t="n"/>
+      <c r="M65" s="39" t="n"/>
+      <c r="N65" s="39" t="n"/>
+      <c r="O65" s="39" t="n"/>
+      <c r="P65" s="39" t="n"/>
+      <c r="Q65" s="39" t="n"/>
+    </row>
+    <row r="66">
+      <c r="B66" s="37" t="n"/>
+      <c r="C66" s="37" t="n"/>
+      <c r="D66" s="37" t="n"/>
+      <c r="E66" s="37" t="n"/>
+      <c r="F66" s="37" t="n"/>
+      <c r="G66" s="37" t="n"/>
+      <c r="H66" s="37" t="n"/>
+      <c r="I66" s="37" t="n"/>
+      <c r="J66" s="37" t="n"/>
+      <c r="K66" s="37" t="n"/>
+      <c r="L66" s="37" t="n"/>
+      <c r="M66" s="37" t="n"/>
+      <c r="N66" s="37" t="n"/>
+      <c r="O66" s="37" t="n"/>
+      <c r="P66" s="37" t="n"/>
+      <c r="Q66" s="37" t="n"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="39" t="n"/>
+      <c r="C67" s="39" t="n"/>
+      <c r="D67" s="39" t="n"/>
+      <c r="E67" s="39" t="n"/>
+      <c r="F67" s="39" t="n"/>
+      <c r="G67" s="39" t="n"/>
+      <c r="H67" s="39" t="n"/>
+      <c r="I67" s="39" t="n"/>
+      <c r="J67" s="39" t="n"/>
+      <c r="K67" s="39" t="n"/>
+      <c r="L67" s="39" t="n"/>
+      <c r="M67" s="39" t="n"/>
+      <c r="N67" s="39" t="n"/>
+      <c r="O67" s="39" t="n"/>
+      <c r="P67" s="39" t="n"/>
+      <c r="Q67" s="39" t="n"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="37" t="n"/>
+      <c r="C68" s="37" t="n"/>
+      <c r="D68" s="37" t="n"/>
+      <c r="E68" s="37" t="n"/>
+      <c r="F68" s="37" t="n"/>
+      <c r="G68" s="37" t="n"/>
+      <c r="H68" s="37" t="n"/>
+      <c r="I68" s="37" t="n"/>
+      <c r="J68" s="37" t="n"/>
+      <c r="K68" s="37" t="n"/>
+      <c r="L68" s="37" t="n"/>
+      <c r="M68" s="37" t="n"/>
+      <c r="N68" s="37" t="n"/>
+      <c r="O68" s="37" t="n"/>
+      <c r="P68" s="37" t="n"/>
+      <c r="Q68" s="37" t="n"/>
+    </row>
+    <row r="69">
+      <c r="B69" s="39" t="n"/>
+      <c r="C69" s="39" t="n"/>
+      <c r="D69" s="39" t="n"/>
+      <c r="E69" s="39" t="n"/>
+      <c r="F69" s="39" t="n"/>
+      <c r="G69" s="39" t="n"/>
+      <c r="H69" s="39" t="n"/>
+      <c r="I69" s="39" t="n"/>
+      <c r="J69" s="39" t="n"/>
+      <c r="K69" s="39" t="n"/>
+      <c r="L69" s="39" t="n"/>
+      <c r="M69" s="39" t="n"/>
+      <c r="N69" s="39" t="n"/>
+      <c r="O69" s="39" t="n"/>
+      <c r="P69" s="39" t="n"/>
+      <c r="Q69" s="39" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="37" t="n"/>
+      <c r="C70" s="37" t="n"/>
+      <c r="D70" s="37" t="n"/>
+      <c r="E70" s="37" t="n"/>
+      <c r="F70" s="37" t="n"/>
+      <c r="G70" s="37" t="n"/>
+      <c r="H70" s="37" t="n"/>
+      <c r="I70" s="37" t="n"/>
+      <c r="J70" s="37" t="n"/>
+      <c r="K70" s="37" t="n"/>
+      <c r="L70" s="37" t="n"/>
+      <c r="M70" s="37" t="n"/>
+      <c r="N70" s="37" t="n"/>
+      <c r="O70" s="37" t="n"/>
+      <c r="P70" s="37" t="n"/>
+      <c r="Q70" s="37" t="n"/>
+    </row>
+    <row r="71">
+      <c r="B71" s="39" t="n"/>
+      <c r="C71" s="39" t="n"/>
+      <c r="D71" s="39" t="n"/>
+      <c r="E71" s="39" t="n"/>
+      <c r="F71" s="39" t="n"/>
+      <c r="G71" s="39" t="n"/>
+      <c r="H71" s="39" t="n"/>
+      <c r="I71" s="39" t="n"/>
+      <c r="J71" s="39" t="n"/>
+      <c r="K71" s="39" t="n"/>
+      <c r="L71" s="39" t="n"/>
+      <c r="M71" s="39" t="n"/>
+      <c r="N71" s="39" t="n"/>
+      <c r="O71" s="39" t="n"/>
+      <c r="P71" s="39" t="n"/>
+      <c r="Q71" s="39" t="n"/>
+    </row>
+    <row r="72">
+      <c r="B72" s="37" t="n"/>
+      <c r="C72" s="37" t="n"/>
+      <c r="D72" s="37" t="n"/>
+      <c r="E72" s="37" t="n"/>
+      <c r="F72" s="37" t="n"/>
+      <c r="G72" s="37" t="n"/>
+      <c r="H72" s="37" t="n"/>
+      <c r="I72" s="37" t="n"/>
+      <c r="J72" s="37" t="n"/>
+      <c r="K72" s="37" t="n"/>
+      <c r="L72" s="37" t="n"/>
+      <c r="M72" s="37" t="n"/>
+      <c r="N72" s="37" t="n"/>
+      <c r="O72" s="37" t="n"/>
+      <c r="P72" s="37" t="n"/>
+      <c r="Q72" s="37" t="n"/>
+    </row>
+    <row r="73">
+      <c r="B73" s="39" t="n"/>
+      <c r="C73" s="39" t="n"/>
+      <c r="D73" s="39" t="n"/>
+      <c r="E73" s="39" t="n"/>
+      <c r="F73" s="39" t="n"/>
+      <c r="G73" s="39" t="n"/>
+      <c r="H73" s="39" t="n"/>
+      <c r="I73" s="39" t="n"/>
+      <c r="J73" s="39" t="n"/>
+      <c r="K73" s="39" t="n"/>
+      <c r="L73" s="39" t="n"/>
+      <c r="M73" s="39" t="n"/>
+      <c r="N73" s="39" t="n"/>
+      <c r="O73" s="39" t="n"/>
+      <c r="P73" s="39" t="n"/>
+      <c r="Q73" s="39" t="n"/>
+    </row>
+    <row r="74">
+      <c r="B74" s="37" t="n"/>
+      <c r="C74" s="37" t="n"/>
+      <c r="D74" s="37" t="n"/>
+      <c r="E74" s="37" t="n"/>
+      <c r="F74" s="37" t="n"/>
+      <c r="G74" s="37" t="n"/>
+      <c r="H74" s="37" t="n"/>
+      <c r="I74" s="37" t="n"/>
+      <c r="J74" s="37" t="n"/>
+      <c r="K74" s="37" t="n"/>
+      <c r="L74" s="37" t="n"/>
+      <c r="M74" s="37" t="n"/>
+      <c r="N74" s="37" t="n"/>
+      <c r="O74" s="37" t="n"/>
+      <c r="P74" s="37" t="n"/>
+      <c r="Q74" s="37" t="n"/>
+    </row>
+    <row r="75">
+      <c r="B75" s="39" t="n"/>
+      <c r="C75" s="39" t="n"/>
+      <c r="D75" s="39" t="n"/>
+      <c r="E75" s="39" t="n"/>
+      <c r="F75" s="39" t="n"/>
+      <c r="G75" s="39" t="n"/>
+      <c r="H75" s="39" t="n"/>
+      <c r="I75" s="39" t="n"/>
+      <c r="J75" s="39" t="n"/>
+      <c r="K75" s="39" t="n"/>
+      <c r="L75" s="39" t="n"/>
+      <c r="M75" s="39" t="n"/>
+      <c r="N75" s="39" t="n"/>
+      <c r="O75" s="39" t="n"/>
+      <c r="P75" s="39" t="n"/>
+      <c r="Q75" s="39" t="n"/>
+    </row>
+    <row r="76">
+      <c r="B76" s="37" t="n"/>
+      <c r="C76" s="37" t="n"/>
+      <c r="D76" s="37" t="n"/>
+      <c r="E76" s="37" t="n"/>
+      <c r="F76" s="37" t="n"/>
+      <c r="G76" s="37" t="n"/>
+      <c r="H76" s="37" t="n"/>
+      <c r="I76" s="37" t="n"/>
+      <c r="J76" s="37" t="n"/>
+      <c r="K76" s="37" t="n"/>
+      <c r="L76" s="37" t="n"/>
+      <c r="M76" s="37" t="n"/>
+      <c r="N76" s="37" t="n"/>
+      <c r="O76" s="37" t="n"/>
+      <c r="P76" s="37" t="n"/>
+      <c r="Q76" s="37" t="n"/>
+    </row>
+    <row r="77">
+      <c r="B77" s="39" t="n"/>
+      <c r="C77" s="39" t="n"/>
+      <c r="D77" s="39" t="n"/>
+      <c r="E77" s="39" t="n"/>
+      <c r="F77" s="39" t="n"/>
+      <c r="G77" s="39" t="n"/>
+      <c r="H77" s="39" t="n"/>
+      <c r="I77" s="39" t="n"/>
+      <c r="J77" s="39" t="n"/>
+      <c r="K77" s="39" t="n"/>
+      <c r="L77" s="39" t="n"/>
+      <c r="M77" s="39" t="n"/>
+      <c r="N77" s="39" t="n"/>
+      <c r="O77" s="39" t="n"/>
+      <c r="P77" s="39" t="n"/>
+      <c r="Q77" s="39" t="n"/>
+    </row>
+    <row r="78">
+      <c r="B78" s="37" t="n"/>
+      <c r="C78" s="37" t="n"/>
+      <c r="D78" s="37" t="n"/>
+      <c r="E78" s="37" t="n"/>
+      <c r="F78" s="37" t="n"/>
+      <c r="G78" s="37" t="n"/>
+      <c r="H78" s="37" t="n"/>
+      <c r="I78" s="37" t="n"/>
+      <c r="J78" s="37" t="n"/>
+      <c r="K78" s="37" t="n"/>
+      <c r="L78" s="37" t="n"/>
+      <c r="M78" s="37" t="n"/>
+      <c r="N78" s="37" t="n"/>
+      <c r="O78" s="37" t="n"/>
+      <c r="P78" s="37" t="n"/>
+      <c r="Q78" s="37" t="n"/>
+    </row>
+    <row r="79">
+      <c r="B79" s="39" t="n"/>
+      <c r="C79" s="39" t="n"/>
+      <c r="D79" s="39" t="n"/>
+      <c r="E79" s="39" t="n"/>
+      <c r="F79" s="39" t="n"/>
+      <c r="G79" s="39" t="n"/>
+      <c r="H79" s="39" t="n"/>
+      <c r="I79" s="39" t="n"/>
+      <c r="J79" s="39" t="n"/>
+      <c r="K79" s="39" t="n"/>
+      <c r="L79" s="39" t="n"/>
+      <c r="M79" s="39" t="n"/>
+      <c r="N79" s="39" t="n"/>
+      <c r="O79" s="39" t="n"/>
+      <c r="P79" s="39" t="n"/>
+      <c r="Q79" s="39" t="n"/>
+    </row>
+    <row r="80">
+      <c r="B80" s="37" t="n"/>
+      <c r="C80" s="37" t="n"/>
+      <c r="D80" s="37" t="n"/>
+      <c r="E80" s="37" t="n"/>
+      <c r="F80" s="37" t="n"/>
+      <c r="G80" s="37" t="n"/>
+      <c r="H80" s="37" t="n"/>
+      <c r="I80" s="37" t="n"/>
+      <c r="J80" s="37" t="n"/>
+      <c r="K80" s="37" t="n"/>
+      <c r="L80" s="37" t="n"/>
+      <c r="M80" s="37" t="n"/>
+      <c r="N80" s="37" t="n"/>
+      <c r="O80" s="37" t="n"/>
+      <c r="P80" s="37" t="n"/>
+      <c r="Q80" s="37" t="n"/>
+    </row>
+    <row r="81">
+      <c r="B81" s="39" t="n"/>
+      <c r="C81" s="39" t="n"/>
+      <c r="D81" s="39" t="n"/>
+      <c r="E81" s="39" t="n"/>
+      <c r="F81" s="39" t="n"/>
+      <c r="G81" s="39" t="n"/>
+      <c r="H81" s="39" t="n"/>
+      <c r="I81" s="39" t="n"/>
+      <c r="J81" s="39" t="n"/>
+      <c r="K81" s="39" t="n"/>
+      <c r="L81" s="39" t="n"/>
+      <c r="M81" s="39" t="n"/>
+      <c r="N81" s="39" t="n"/>
+      <c r="O81" s="39" t="n"/>
+      <c r="P81" s="39" t="n"/>
+      <c r="Q81" s="39" t="n"/>
+    </row>
+    <row r="82">
+      <c r="B82" s="37" t="n"/>
+      <c r="C82" s="37" t="n"/>
+      <c r="D82" s="37" t="n"/>
+      <c r="E82" s="37" t="n"/>
+      <c r="F82" s="37" t="n"/>
+      <c r="G82" s="37" t="n"/>
+      <c r="H82" s="37" t="n"/>
+      <c r="I82" s="37" t="n"/>
+      <c r="J82" s="37" t="n"/>
+      <c r="K82" s="37" t="n"/>
+      <c r="L82" s="37" t="n"/>
+      <c r="M82" s="37" t="n"/>
+      <c r="N82" s="37" t="n"/>
+      <c r="O82" s="37" t="n"/>
+      <c r="P82" s="37" t="n"/>
+      <c r="Q82" s="37" t="n"/>
+    </row>
+    <row r="83">
+      <c r="B83" s="39" t="n"/>
+      <c r="C83" s="39" t="n"/>
+      <c r="D83" s="39" t="n"/>
+      <c r="E83" s="39" t="n"/>
+      <c r="F83" s="39" t="n"/>
+      <c r="G83" s="39" t="n"/>
+      <c r="H83" s="39" t="n"/>
+      <c r="I83" s="39" t="n"/>
+      <c r="J83" s="39" t="n"/>
+      <c r="K83" s="39" t="n"/>
+      <c r="L83" s="39" t="n"/>
+      <c r="M83" s="39" t="n"/>
+      <c r="N83" s="39" t="n"/>
+      <c r="O83" s="39" t="n"/>
+      <c r="P83" s="39" t="n"/>
+      <c r="Q83" s="39" t="n"/>
+    </row>
+    <row r="84">
+      <c r="B84" s="37" t="n"/>
+      <c r="C84" s="37" t="n"/>
+      <c r="D84" s="37" t="n"/>
+      <c r="E84" s="37" t="n"/>
+      <c r="F84" s="37" t="n"/>
+      <c r="G84" s="37" t="n"/>
+      <c r="H84" s="37" t="n"/>
+      <c r="I84" s="37" t="n"/>
+      <c r="J84" s="37" t="n"/>
+      <c r="K84" s="37" t="n"/>
+      <c r="L84" s="37" t="n"/>
+      <c r="M84" s="37" t="n"/>
+      <c r="N84" s="37" t="n"/>
+      <c r="O84" s="37" t="n"/>
+      <c r="P84" s="37" t="n"/>
+      <c r="Q84" s="37" t="n"/>
+    </row>
+    <row r="85">
+      <c r="B85" s="39" t="n"/>
+      <c r="C85" s="39" t="n"/>
+      <c r="D85" s="39" t="n"/>
+      <c r="E85" s="39" t="n"/>
+      <c r="F85" s="39" t="n"/>
+      <c r="G85" s="39" t="n"/>
+      <c r="H85" s="39" t="n"/>
+      <c r="I85" s="39" t="n"/>
+      <c r="J85" s="39" t="n"/>
+      <c r="K85" s="39" t="n"/>
+      <c r="L85" s="39" t="n"/>
+      <c r="M85" s="39" t="n"/>
+      <c r="N85" s="39" t="n"/>
+      <c r="O85" s="39" t="n"/>
+      <c r="P85" s="39" t="n"/>
+      <c r="Q85" s="39" t="n"/>
+    </row>
+    <row r="86">
+      <c r="B86" s="37" t="n"/>
+      <c r="C86" s="37" t="n"/>
+      <c r="D86" s="37" t="n"/>
+      <c r="E86" s="37" t="n"/>
+      <c r="F86" s="37" t="n"/>
+      <c r="G86" s="37" t="n"/>
+      <c r="H86" s="37" t="n"/>
+      <c r="I86" s="37" t="n"/>
+      <c r="J86" s="37" t="n"/>
+      <c r="K86" s="37" t="n"/>
+      <c r="L86" s="37" t="n"/>
+      <c r="M86" s="37" t="n"/>
+      <c r="N86" s="37" t="n"/>
+      <c r="O86" s="37" t="n"/>
+      <c r="P86" s="37" t="n"/>
+      <c r="Q86" s="37" t="n"/>
+    </row>
+    <row r="87">
+      <c r="B87" s="39" t="n"/>
+      <c r="C87" s="39" t="n"/>
+      <c r="D87" s="39" t="n"/>
+      <c r="E87" s="39" t="n"/>
+      <c r="F87" s="39" t="n"/>
+      <c r="G87" s="39" t="n"/>
+      <c r="H87" s="39" t="n"/>
+      <c r="I87" s="39" t="n"/>
+      <c r="J87" s="39" t="n"/>
+      <c r="K87" s="39" t="n"/>
+      <c r="L87" s="39" t="n"/>
+      <c r="M87" s="39" t="n"/>
+      <c r="N87" s="39" t="n"/>
+      <c r="O87" s="39" t="n"/>
+      <c r="P87" s="39" t="n"/>
+      <c r="Q87" s="39" t="n"/>
+    </row>
+    <row r="88">
+      <c r="B88" s="37" t="n"/>
+      <c r="C88" s="37" t="n"/>
+      <c r="D88" s="37" t="n"/>
+      <c r="E88" s="37" t="n"/>
+      <c r="F88" s="37" t="n"/>
+      <c r="G88" s="37" t="n"/>
+      <c r="H88" s="37" t="n"/>
+      <c r="I88" s="37" t="n"/>
+      <c r="J88" s="37" t="n"/>
+      <c r="K88" s="37" t="n"/>
+      <c r="L88" s="37" t="n"/>
+      <c r="M88" s="37" t="n"/>
+      <c r="N88" s="37" t="n"/>
+      <c r="O88" s="37" t="n"/>
+      <c r="P88" s="37" t="n"/>
+      <c r="Q88" s="37" t="n"/>
+    </row>
+    <row r="89">
+      <c r="B89" s="39" t="n"/>
+      <c r="C89" s="39" t="n"/>
+      <c r="D89" s="39" t="n"/>
+      <c r="E89" s="39" t="n"/>
+      <c r="F89" s="39" t="n"/>
+      <c r="G89" s="39" t="n"/>
+      <c r="H89" s="39" t="n"/>
+      <c r="I89" s="39" t="n"/>
+      <c r="J89" s="39" t="n"/>
+      <c r="K89" s="39" t="n"/>
+      <c r="L89" s="39" t="n"/>
+      <c r="M89" s="39" t="n"/>
+      <c r="N89" s="39" t="n"/>
+      <c r="O89" s="39" t="n"/>
+      <c r="P89" s="39" t="n"/>
+      <c r="Q89" s="39" t="n"/>
+    </row>
+    <row r="90">
+      <c r="B90" s="37" t="n"/>
+      <c r="C90" s="37" t="n"/>
+      <c r="D90" s="37" t="n"/>
+      <c r="E90" s="37" t="n"/>
+      <c r="F90" s="37" t="n"/>
+      <c r="G90" s="37" t="n"/>
+      <c r="H90" s="37" t="n"/>
+      <c r="I90" s="37" t="n"/>
+      <c r="J90" s="37" t="n"/>
+      <c r="K90" s="37" t="n"/>
+      <c r="L90" s="37" t="n"/>
+      <c r="M90" s="37" t="n"/>
+      <c r="N90" s="37" t="n"/>
+      <c r="O90" s="37" t="n"/>
+      <c r="P90" s="37" t="n"/>
+      <c r="Q90" s="37" t="n"/>
+    </row>
+    <row r="91">
+      <c r="B91" s="39" t="n"/>
+      <c r="C91" s="39" t="n"/>
+      <c r="D91" s="39" t="n"/>
+      <c r="E91" s="39" t="n"/>
+      <c r="F91" s="39" t="n"/>
+      <c r="G91" s="39" t="n"/>
+      <c r="H91" s="39" t="n"/>
+      <c r="I91" s="39" t="n"/>
+      <c r="J91" s="39" t="n"/>
+      <c r="K91" s="39" t="n"/>
+      <c r="L91" s="39" t="n"/>
+      <c r="M91" s="39" t="n"/>
+      <c r="N91" s="39" t="n"/>
+      <c r="O91" s="39" t="n"/>
+      <c r="P91" s="39" t="n"/>
+      <c r="Q91" s="39" t="n"/>
+    </row>
+    <row r="92">
+      <c r="B92" s="37" t="n"/>
+      <c r="C92" s="37" t="n"/>
+      <c r="D92" s="37" t="n"/>
+      <c r="E92" s="37" t="n"/>
+      <c r="F92" s="37" t="n"/>
+      <c r="G92" s="37" t="n"/>
+      <c r="H92" s="37" t="n"/>
+      <c r="I92" s="37" t="n"/>
+      <c r="J92" s="37" t="n"/>
+      <c r="K92" s="37" t="n"/>
+      <c r="L92" s="37" t="n"/>
+      <c r="M92" s="37" t="n"/>
+      <c r="N92" s="37" t="n"/>
+      <c r="O92" s="37" t="n"/>
+      <c r="P92" s="37" t="n"/>
+      <c r="Q92" s="37" t="n"/>
+    </row>
+    <row r="93">
+      <c r="B93" s="39" t="n"/>
+      <c r="C93" s="39" t="n"/>
+      <c r="D93" s="39" t="n"/>
+      <c r="E93" s="39" t="n"/>
+      <c r="F93" s="39" t="n"/>
+      <c r="G93" s="39" t="n"/>
+      <c r="H93" s="39" t="n"/>
+      <c r="I93" s="39" t="n"/>
+      <c r="J93" s="39" t="n"/>
+      <c r="K93" s="39" t="n"/>
+      <c r="L93" s="39" t="n"/>
+      <c r="M93" s="39" t="n"/>
+      <c r="N93" s="39" t="n"/>
+      <c r="O93" s="39" t="n"/>
+      <c r="P93" s="39" t="n"/>
+      <c r="Q93" s="39" t="n"/>
+    </row>
+    <row r="94">
+      <c r="B94" s="37" t="n"/>
+      <c r="C94" s="37" t="n"/>
+      <c r="D94" s="37" t="n"/>
+      <c r="E94" s="37" t="n"/>
+      <c r="F94" s="37" t="n"/>
+      <c r="G94" s="37" t="n"/>
+      <c r="H94" s="37" t="n"/>
+      <c r="I94" s="37" t="n"/>
+      <c r="J94" s="37" t="n"/>
+      <c r="K94" s="37" t="n"/>
+      <c r="L94" s="37" t="n"/>
+      <c r="M94" s="37" t="n"/>
+      <c r="N94" s="37" t="n"/>
+      <c r="O94" s="37" t="n"/>
+      <c r="P94" s="37" t="n"/>
+      <c r="Q94" s="37" t="n"/>
+    </row>
+    <row r="95">
+      <c r="B95" s="39" t="n"/>
+      <c r="C95" s="39" t="n"/>
+      <c r="D95" s="39" t="n"/>
+      <c r="E95" s="39" t="n"/>
+      <c r="F95" s="39" t="n"/>
+      <c r="G95" s="39" t="n"/>
+      <c r="H95" s="39" t="n"/>
+      <c r="I95" s="39" t="n"/>
+      <c r="J95" s="39" t="n"/>
+      <c r="K95" s="39" t="n"/>
+      <c r="L95" s="39" t="n"/>
+      <c r="M95" s="39" t="n"/>
+      <c r="N95" s="39" t="n"/>
+      <c r="O95" s="39" t="n"/>
+      <c r="P95" s="39" t="n"/>
+      <c r="Q95" s="39" t="n"/>
+    </row>
+    <row r="96">
+      <c r="B96" s="37" t="n"/>
+      <c r="C96" s="37" t="n"/>
+      <c r="D96" s="37" t="n"/>
+      <c r="E96" s="37" t="n"/>
+      <c r="F96" s="37" t="n"/>
+      <c r="G96" s="37" t="n"/>
+      <c r="H96" s="37" t="n"/>
+      <c r="I96" s="37" t="n"/>
+      <c r="J96" s="37" t="n"/>
+      <c r="K96" s="37" t="n"/>
+      <c r="L96" s="37" t="n"/>
+      <c r="M96" s="37" t="n"/>
+      <c r="N96" s="37" t="n"/>
+      <c r="O96" s="37" t="n"/>
+      <c r="P96" s="37" t="n"/>
+      <c r="Q96" s="37" t="n"/>
+    </row>
+    <row r="97">
+      <c r="B97" s="39" t="n"/>
+      <c r="C97" s="39" t="n"/>
+      <c r="D97" s="39" t="n"/>
+      <c r="E97" s="39" t="n"/>
+      <c r="F97" s="39" t="n"/>
+      <c r="G97" s="39" t="n"/>
+      <c r="H97" s="39" t="n"/>
+      <c r="I97" s="39" t="n"/>
+      <c r="J97" s="39" t="n"/>
+      <c r="K97" s="39" t="n"/>
+      <c r="L97" s="39" t="n"/>
+      <c r="M97" s="39" t="n"/>
+      <c r="N97" s="39" t="n"/>
+      <c r="O97" s="39" t="n"/>
+      <c r="P97" s="39" t="n"/>
+      <c r="Q97" s="39" t="n"/>
+    </row>
+    <row r="98">
+      <c r="B98" s="37" t="n"/>
+      <c r="C98" s="37" t="n"/>
+      <c r="D98" s="37" t="n"/>
+      <c r="E98" s="37" t="n"/>
+      <c r="F98" s="37" t="n"/>
+      <c r="G98" s="37" t="n"/>
+      <c r="H98" s="37" t="n"/>
+      <c r="I98" s="37" t="n"/>
+      <c r="J98" s="37" t="n"/>
+      <c r="K98" s="37" t="n"/>
+      <c r="L98" s="37" t="n"/>
+      <c r="M98" s="37" t="n"/>
+      <c r="N98" s="37" t="n"/>
+      <c r="O98" s="37" t="n"/>
+      <c r="P98" s="37" t="n"/>
+      <c r="Q98" s="37" t="n"/>
+    </row>
+    <row r="99">
+      <c r="B99" s="39" t="n"/>
+      <c r="C99" s="39" t="n"/>
+      <c r="D99" s="39" t="n"/>
+      <c r="E99" s="39" t="n"/>
+      <c r="F99" s="39" t="n"/>
+      <c r="G99" s="39" t="n"/>
+      <c r="H99" s="39" t="n"/>
+      <c r="I99" s="39" t="n"/>
+      <c r="J99" s="39" t="n"/>
+      <c r="K99" s="39" t="n"/>
+      <c r="L99" s="39" t="n"/>
+      <c r="M99" s="39" t="n"/>
+      <c r="N99" s="39" t="n"/>
+      <c r="O99" s="39" t="n"/>
+      <c r="P99" s="39" t="n"/>
+      <c r="Q99" s="39" t="n"/>
+    </row>
+    <row r="100">
+      <c r="B100" s="37" t="n"/>
+      <c r="C100" s="37" t="n"/>
+      <c r="D100" s="37" t="n"/>
+      <c r="E100" s="37" t="n"/>
+      <c r="F100" s="37" t="n"/>
+      <c r="G100" s="37" t="n"/>
+      <c r="H100" s="37" t="n"/>
+      <c r="I100" s="37" t="n"/>
+      <c r="J100" s="37" t="n"/>
+      <c r="K100" s="37" t="n"/>
+      <c r="L100" s="37" t="n"/>
+      <c r="M100" s="37" t="n"/>
+      <c r="N100" s="37" t="n"/>
+      <c r="O100" s="37" t="n"/>
+      <c r="P100" s="37" t="n"/>
+      <c r="Q100" s="37" t="n"/>
+    </row>
+    <row r="101">
+      <c r="B101" s="39" t="n"/>
+      <c r="C101" s="39" t="n"/>
+      <c r="D101" s="39" t="n"/>
+      <c r="E101" s="39" t="n"/>
+      <c r="F101" s="39" t="n"/>
+      <c r="G101" s="39" t="n"/>
+      <c r="H101" s="39" t="n"/>
+      <c r="I101" s="39" t="n"/>
+      <c r="J101" s="39" t="n"/>
+      <c r="K101" s="39" t="n"/>
+      <c r="L101" s="39" t="n"/>
+      <c r="M101" s="39" t="n"/>
+      <c r="N101" s="39" t="n"/>
+      <c r="O101" s="39" t="n"/>
+      <c r="P101" s="39" t="n"/>
+      <c r="Q101" s="39" t="n"/>
+    </row>
+    <row r="102">
+      <c r="B102" s="37" t="n"/>
+      <c r="C102" s="37" t="n"/>
+      <c r="D102" s="37" t="n"/>
+      <c r="E102" s="37" t="n"/>
+      <c r="F102" s="37" t="n"/>
+      <c r="G102" s="37" t="n"/>
+      <c r="H102" s="37" t="n"/>
+      <c r="I102" s="37" t="n"/>
+      <c r="J102" s="37" t="n"/>
+      <c r="K102" s="37" t="n"/>
+      <c r="L102" s="37" t="n"/>
+      <c r="M102" s="37" t="n"/>
+      <c r="N102" s="37" t="n"/>
+      <c r="O102" s="37" t="n"/>
+      <c r="P102" s="37" t="n"/>
+      <c r="Q102" s="37" t="n"/>
+    </row>
+    <row r="103">
+      <c r="B103" s="39" t="n"/>
+      <c r="C103" s="39" t="n"/>
+      <c r="D103" s="39" t="n"/>
+      <c r="E103" s="39" t="n"/>
+      <c r="F103" s="39" t="n"/>
+      <c r="G103" s="39" t="n"/>
+      <c r="H103" s="39" t="n"/>
+      <c r="I103" s="39" t="n"/>
+      <c r="J103" s="39" t="n"/>
+      <c r="K103" s="39" t="n"/>
+      <c r="L103" s="39" t="n"/>
+      <c r="M103" s="39" t="n"/>
+      <c r="N103" s="39" t="n"/>
+      <c r="O103" s="39" t="n"/>
+      <c r="P103" s="39" t="n"/>
+      <c r="Q103" s="39" t="n"/>
+    </row>
+    <row r="104">
+      <c r="B104" s="37" t="n"/>
+      <c r="C104" s="37" t="n"/>
+      <c r="D104" s="37" t="n"/>
+      <c r="E104" s="37" t="n"/>
+      <c r="F104" s="37" t="n"/>
+      <c r="G104" s="37" t="n"/>
+      <c r="H104" s="37" t="n"/>
+      <c r="I104" s="37" t="n"/>
+      <c r="J104" s="37" t="n"/>
+      <c r="K104" s="37" t="n"/>
+      <c r="L104" s="37" t="n"/>
+      <c r="M104" s="37" t="n"/>
+      <c r="N104" s="37" t="n"/>
+      <c r="O104" s="37" t="n"/>
+      <c r="P104" s="37" t="n"/>
+      <c r="Q104" s="37" t="n"/>
+    </row>
+    <row r="107">
+      <c r="B107" s="16" t="inlineStr">
+        <is>
+          <t>💡 Tip: Select Row 4 → Copy → Select target row → Paste Special → Values Only. This freezes the current analysis as a permanent record.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B1:O1"/>
-    <mergeCell ref="B2:O2"/>
+  <mergeCells count="3">
+    <mergeCell ref="B2:Q2"/>
+    <mergeCell ref="B107:Q107"/>
+    <mergeCell ref="B1:Q1"/>
   </mergeCells>
-  <conditionalFormatting sqref="L4:L55">
+  <conditionalFormatting sqref="L4:L105">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>1.67</formula>
     </cfRule>
@@ -13847,7 +14892,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K4:K55">
+  <conditionalFormatting sqref="M4:M105">
     <cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" dxfId="0">
       <formula>1.67</formula>
     </cfRule>
@@ -13870,11 +14915,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B52"/>
+  <dimension ref="B1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13885,324 +14933,998 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="58" t="inlineStr"/>
+      <c r="B3" s="58" t="inlineStr">
+        <is>
+          <t>📏 Cpk / Capability Thresholds</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" s="59" t="inlineStr">
         <is>
-          <t>How to Use This Workbook</t>
+          <t>Cpk Range</t>
+        </is>
+      </c>
+      <c r="C4" s="59" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="D4" s="59" t="inlineStr">
+        <is>
+          <t>PPM (approx.)</t>
+        </is>
+      </c>
+      <c r="E4" s="59" t="inlineStr">
+        <is>
+          <t>Action</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="58" t="inlineStr">
-        <is>
-          <t>1. Enter specifications (Tₘ, LSL, USL) in the Analysis sheet (blue cells)</t>
+      <c r="B5" s="60" t="inlineStr">
+        <is>
+          <t>&lt; 1.00</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>❌ Not Capable</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>&gt; 2,700</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr">
+        <is>
+          <t>Process redesign or tighter controls needed</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="58" t="inlineStr">
-        <is>
-          <t>2. Choose Mode: 'Enter Manually' or 'Use Data Worksheet' (dropdown in C10)</t>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>1.00 – 1.33</t>
+        </is>
+      </c>
+      <c r="C6" s="61" t="inlineStr">
+        <is>
+          <t>⚠️ Marginal</t>
+        </is>
+      </c>
+      <c r="D6" s="61" t="inlineStr">
+        <is>
+          <t>63 – 2,700</t>
+        </is>
+      </c>
+      <c r="E6" s="61" t="inlineStr">
+        <is>
+          <t>Improvement required, monitor closely</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="58" t="inlineStr">
-        <is>
-          <t>3. If Manual: enter x̄, σ, n directly in the Analysis sheet</t>
+      <c r="B7" s="60" t="inlineStr">
+        <is>
+          <t>1.33 – 1.67</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>✅ Capable</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>0.6 – 63</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="inlineStr">
+        <is>
+          <t>Meets most industry standards</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="58" t="inlineStr">
-        <is>
-          <t>4. If Worksheet: enter part data in the Data sheet — mean &amp; σ auto-link</t>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>1.67 – 2.00</t>
+        </is>
+      </c>
+      <c r="C8" s="61" t="inlineStr">
+        <is>
+          <t>✅ Highly Capable</t>
+        </is>
+      </c>
+      <c r="D8" s="61" t="inlineStr">
+        <is>
+          <t>&lt; 0.6</t>
+        </is>
+      </c>
+      <c r="E8" s="61" t="inlineStr">
+        <is>
+          <t>Meets automotive/safety-critical</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="58" t="inlineStr">
-        <is>
-          <t>5. All results, probability, hypothesis test, and verdict update INSTANTLY</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="58" t="inlineStr">
-        <is>
-          <t>6. View charts in the Charts sheet (bell curve + capability bars)</t>
+      <c r="B9" s="60" t="inlineStr">
+        <is>
+          <t>≥ 2.00</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>🏆 Six Sigma</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>&lt; 0.002</t>
+        </is>
+      </c>
+      <c r="E9" s="61" t="inlineStr">
+        <is>
+          <t>World-class capability</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="58" t="inlineStr">
         <is>
-          <t>7. To save a run: go to History sheet, copy Row 4, paste as VALUES into Row 5+</t>
+          <t>📊 Sigma Level &amp; PPM Table</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="58" t="inlineStr"/>
+      <c r="B12" s="59" t="inlineStr">
+        <is>
+          <t>Sigma Level</t>
+        </is>
+      </c>
+      <c r="C12" s="59" t="inlineStr">
+        <is>
+          <t>Yield (%)</t>
+        </is>
+      </c>
+      <c r="D12" s="59" t="inlineStr">
+        <is>
+          <t>DPMO (PPM)</t>
+        </is>
+      </c>
+      <c r="E12" s="59" t="inlineStr">
+        <is>
+          <t>Cpk</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="B13" s="59" t="inlineStr">
-        <is>
-          <t>Core Capability Formulas</t>
+      <c r="B13" s="60" t="inlineStr">
+        <is>
+          <t>1σ</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>30.85%</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>691,462</t>
+        </is>
+      </c>
+      <c r="E13" s="61" t="inlineStr">
+        <is>
+          <t>0.33</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Cp = (USL − LSL) / 6σ  — Potential capability if process is perfectly centered</t>
+      <c r="B14" s="60" t="inlineStr">
+        <is>
+          <t>2σ</t>
+        </is>
+      </c>
+      <c r="C14" s="61" t="inlineStr">
+        <is>
+          <t>69.15%</t>
+        </is>
+      </c>
+      <c r="D14" s="61" t="inlineStr">
+        <is>
+          <t>308,538</t>
+        </is>
+      </c>
+      <c r="E14" s="61" t="inlineStr">
+        <is>
+          <t>0.67</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Cpk = min[(USL − x̄) / 3σ,  (x̄ − LSL) / 3σ]  — Actual capability with centering error</t>
+      <c r="B15" s="60" t="inlineStr">
+        <is>
+          <t>3σ</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>93.32%</t>
+        </is>
+      </c>
+      <c r="D15" s="61" t="inlineStr">
+        <is>
+          <t>66,807</t>
+        </is>
+      </c>
+      <c r="E15" s="61" t="inlineStr">
+        <is>
+          <t>1.00</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Required Shift (Δ) = Tₘ − x̄  — How far to adjust the process mean</t>
+      <c r="B16" s="60" t="inlineStr">
+        <is>
+          <t>4σ</t>
+        </is>
+      </c>
+      <c r="C16" s="61" t="inlineStr">
+        <is>
+          <t>99.3790%</t>
+        </is>
+      </c>
+      <c r="D16" s="61" t="inlineStr">
+        <is>
+          <t>6,210</t>
+        </is>
+      </c>
+      <c r="E16" s="61" t="inlineStr">
+        <is>
+          <t>1.33</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Required Tolerance = Target Index × 6σ  — Minimum tolerance band needed</t>
+      <c r="B17" s="60" t="inlineStr">
+        <is>
+          <t>5σ</t>
+        </is>
+      </c>
+      <c r="C17" s="61" t="inlineStr">
+        <is>
+          <t>99.97670%</t>
+        </is>
+      </c>
+      <c r="D17" s="61" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="E17" s="61" t="inlineStr">
+        <is>
+          <t>1.67</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="58" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="59" t="inlineStr">
-        <is>
-          <t>Capability Index Interpretation (Automotive Standards)</t>
+      <c r="B18" s="60" t="inlineStr">
+        <is>
+          <t>6σ</t>
+        </is>
+      </c>
+      <c r="C18" s="61" t="inlineStr">
+        <is>
+          <t>99.99966%</t>
+        </is>
+      </c>
+      <c r="D18" s="61" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="E18" s="61" t="inlineStr">
+        <is>
+          <t>2.00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cpk ≥ 1.67  →  ✅ GOOD — Capable (standard automotive target)</t>
+          <t>🔬 Core SPC Formulas</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1.33 ≤ Cpk &lt; 1.67  →  ⚠ ACCEPTABLE — Meets minimum but below target</t>
-        </is>
-      </c>
+      <c r="B21" s="59" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="C21" s="59" t="inlineStr">
+        <is>
+          <t>Expression</t>
+        </is>
+      </c>
+      <c r="D21" s="59" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="E21" s="59" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="B22" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1.00 ≤ Cpk &lt; 1.33  →  ⚠ MARGINAL — High risk, improvement needed</t>
-        </is>
-      </c>
+      <c r="B22" s="60" t="inlineStr">
+        <is>
+          <t>Cp</t>
+        </is>
+      </c>
+      <c r="C22" s="61" t="inlineStr">
+        <is>
+          <t>(USL − LSL) / 6σ</t>
+        </is>
+      </c>
+      <c r="D22" s="61" t="inlineStr">
+        <is>
+          <t>Potential capability (centered)</t>
+        </is>
+      </c>
+      <c r="E22" s="61" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="B23" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Cpk &lt; 1.00  →  ❌ NOT CAPABLE — Produces significant defects</t>
-        </is>
-      </c>
+      <c r="B23" s="60" t="inlineStr">
+        <is>
+          <t>Cpk</t>
+        </is>
+      </c>
+      <c r="C23" s="61" t="inlineStr">
+        <is>
+          <t>min[(USL − x̄)/3σ, (x̄ − LSL)/3σ]</t>
+        </is>
+      </c>
+      <c r="D23" s="61" t="inlineStr">
+        <is>
+          <t>Actual capability (with shift)</t>
+        </is>
+      </c>
+      <c r="E23" s="61" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="B24" s="58" t="inlineStr"/>
+      <c r="B24" s="60" t="inlineStr">
+        <is>
+          <t>Pp</t>
+        </is>
+      </c>
+      <c r="C24" s="61" t="inlineStr">
+        <is>
+          <t>(USL − LSL) / 6σ_overall</t>
+        </is>
+      </c>
+      <c r="D24" s="61" t="inlineStr">
+        <is>
+          <t>Long-term potential performance</t>
+        </is>
+      </c>
+      <c r="E24" s="61" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="B25" s="59" t="inlineStr">
-        <is>
-          <t>Probability &amp; PPM</t>
-        </is>
-      </c>
+      <c r="B25" s="60" t="inlineStr">
+        <is>
+          <t>Ppk</t>
+        </is>
+      </c>
+      <c r="C25" s="61" t="inlineStr">
+        <is>
+          <t>min[(USL − x̄)/3σ_overall, (x̄ − LSL)/3σ_overall]</t>
+        </is>
+      </c>
+      <c r="D25" s="61" t="inlineStr">
+        <is>
+          <t>Long-term actual performance</t>
+        </is>
+      </c>
+      <c r="E25" s="61" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="B26" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  P(x &gt; USL) — Probability a part exceeds upper spec limit</t>
-        </is>
-      </c>
+      <c r="B26" s="60" t="inlineStr">
+        <is>
+          <t>Shift (Δ)</t>
+        </is>
+      </c>
+      <c r="C26" s="61" t="inlineStr">
+        <is>
+          <t>Tₘ − x̄</t>
+        </is>
+      </c>
+      <c r="D26" s="61" t="inlineStr">
+        <is>
+          <t>Required mean adjustment</t>
+        </is>
+      </c>
+      <c r="E26" s="61" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="B27" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  P(x &lt; LSL) — Probability a part falls below lower spec limit</t>
-        </is>
-      </c>
+      <c r="B27" s="60" t="inlineStr">
+        <is>
+          <t>Z-score</t>
+        </is>
+      </c>
+      <c r="C27" s="61" t="inlineStr">
+        <is>
+          <t>(x̄ − Tₘ) / (σ / √n)</t>
+        </is>
+      </c>
+      <c r="D27" s="61" t="inlineStr">
+        <is>
+          <t>Hypothesis test statistic</t>
+        </is>
+      </c>
+      <c r="E27" s="61" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="B28" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PPM = Probability × 1,000,000 — Parts Per Million defective</t>
-        </is>
-      </c>
+      <c r="B28" s="60" t="inlineStr">
+        <is>
+          <t>UCL</t>
+        </is>
+      </c>
+      <c r="C28" s="61" t="inlineStr">
+        <is>
+          <t>x̄ + 3σ</t>
+        </is>
+      </c>
+      <c r="D28" s="61" t="inlineStr">
+        <is>
+          <t>Upper control limit</t>
+        </is>
+      </c>
+      <c r="E28" s="61" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="B29" s="58" t="inlineStr"/>
+      <c r="B29" s="60" t="inlineStr">
+        <is>
+          <t>LCL</t>
+        </is>
+      </c>
+      <c r="C29" s="61" t="inlineStr">
+        <is>
+          <t>x̄ − 3σ</t>
+        </is>
+      </c>
+      <c r="D29" s="61" t="inlineStr">
+        <is>
+          <t>Lower control limit</t>
+        </is>
+      </c>
+      <c r="E29" s="61" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="B30" s="59" t="inlineStr">
-        <is>
-          <t>Hypothesis Testing</t>
-        </is>
-      </c>
+      <c r="B30" s="60" t="inlineStr">
+        <is>
+          <t>MR̄</t>
+        </is>
+      </c>
+      <c r="C30" s="61" t="inlineStr">
+        <is>
+          <t>Σ|Xᵢ − Xᵢ₋₁| / (n−1)</t>
+        </is>
+      </c>
+      <c r="D30" s="61" t="inlineStr">
+        <is>
+          <t>Average moving range</t>
+        </is>
+      </c>
+      <c r="E30" s="61" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="B31" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  H₀: μ = Tₘ (process is on target)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Z = (x̄ − Tₘ) / (σ / √n)</t>
-        </is>
-      </c>
+      <c r="B31" s="60" t="inlineStr">
+        <is>
+          <t>MR UCL</t>
+        </is>
+      </c>
+      <c r="C31" s="61" t="inlineStr">
+        <is>
+          <t>3.267 × MR̄</t>
+        </is>
+      </c>
+      <c r="D31" s="61" t="inlineStr">
+        <is>
+          <t>MR chart upper control limit</t>
+        </is>
+      </c>
+      <c r="E31" s="61" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="B33" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  p-value &lt; α → Reject H₀ → Significant shift detected</t>
+          <t>🎯 Control Chart Zones (I-MR)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  p-value ≥ α → Fail to Reject H₀ → No significant shift</t>
+      <c r="B34" s="59" t="inlineStr">
+        <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="C34" s="59" t="inlineStr">
+        <is>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="D34" s="59" t="inlineStr">
+        <is>
+          <t>Expected %</t>
+        </is>
+      </c>
+      <c r="E34" s="59" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Two-Sided: tests if mean differs in either direction</t>
+      <c r="B35" s="60" t="inlineStr">
+        <is>
+          <t>Zone C</t>
+        </is>
+      </c>
+      <c r="C35" s="61" t="inlineStr">
+        <is>
+          <t>x̄ ± 1σ</t>
+        </is>
+      </c>
+      <c r="D35" s="61" t="inlineStr">
+        <is>
+          <t>68.27%</t>
+        </is>
+      </c>
+      <c r="E35" s="61" t="inlineStr">
+        <is>
+          <t>Normal — process in control</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Upper-Sided: tests if mean is significantly above target</t>
+      <c r="B36" s="60" t="inlineStr">
+        <is>
+          <t>Zone B</t>
+        </is>
+      </c>
+      <c r="C36" s="61" t="inlineStr">
+        <is>
+          <t>x̄ ± 1σ to ± 2σ</t>
+        </is>
+      </c>
+      <c r="D36" s="61" t="inlineStr">
+        <is>
+          <t>27.18%</t>
+        </is>
+      </c>
+      <c r="E36" s="61" t="inlineStr">
+        <is>
+          <t>Caution — monitor</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Lower-Sided: tests if mean is significantly below target</t>
+      <c r="B37" s="60" t="inlineStr">
+        <is>
+          <t>Zone A</t>
+        </is>
+      </c>
+      <c r="C37" s="61" t="inlineStr">
+        <is>
+          <t>x̄ ± 2σ to ± 3σ</t>
+        </is>
+      </c>
+      <c r="D37" s="61" t="inlineStr">
+        <is>
+          <t>4.28%</t>
+        </is>
+      </c>
+      <c r="E37" s="61" t="inlineStr">
+        <is>
+          <t>Warning — investigate</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="58" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="59" t="inlineStr">
-        <is>
-          <t>Robustness Assessment</t>
+      <c r="B38" s="60" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="C38" s="61" t="inlineStr">
+        <is>
+          <t>Beyond ± 3σ</t>
+        </is>
+      </c>
+      <c r="D38" s="61" t="inlineStr">
+        <is>
+          <t>0.27%</t>
+        </is>
+      </c>
+      <c r="E38" s="61" t="inlineStr">
+        <is>
+          <t>Out of Control — action required</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ROBUST: ±4σ spread contained within specification limits</t>
+          <t>⚠️ Western Electric Rules</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MARGINAL: ±3σ contained but ±4σ is NOT — low tolerance for future shifts</t>
-        </is>
-      </c>
+      <c r="B41" s="59" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="C41" s="59" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D41" s="59" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="E41" s="59" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="B42" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NOT ROBUST: ±3σ breaches specification limits</t>
-        </is>
-      </c>
+      <c r="B42" s="60" t="inlineStr">
+        <is>
+          <t>Rule 1</t>
+        </is>
+      </c>
+      <c r="C42" s="61" t="inlineStr">
+        <is>
+          <t>Any single point beyond ±3σ</t>
+        </is>
+      </c>
+      <c r="D42" s="61" t="inlineStr">
+        <is>
+          <t>Out of Control</t>
+        </is>
+      </c>
+      <c r="E42" s="61" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="B43" s="58" t="inlineStr"/>
+      <c r="B43" s="60" t="inlineStr">
+        <is>
+          <t>Rule 2</t>
+        </is>
+      </c>
+      <c r="C43" s="61" t="inlineStr">
+        <is>
+          <t>2 of 3 consecutive points beyond ±2σ (same side)</t>
+        </is>
+      </c>
+      <c r="D43" s="61" t="inlineStr">
+        <is>
+          <t>Process shift warning</t>
+        </is>
+      </c>
+      <c r="E43" s="61" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="B44" s="59" t="inlineStr">
-        <is>
-          <t>Spread Metrics</t>
-        </is>
-      </c>
+      <c r="B44" s="60" t="inlineStr">
+        <is>
+          <t>Rule 3</t>
+        </is>
+      </c>
+      <c r="C44" s="61" t="inlineStr">
+        <is>
+          <t>4 of 5 consecutive points beyond ±1σ (same side)</t>
+        </is>
+      </c>
+      <c r="D44" s="61" t="inlineStr">
+        <is>
+          <t>Developing trend</t>
+        </is>
+      </c>
+      <c r="E44" s="61" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="B45" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  6σ Spread — Contains ~99.73% of process output (±3σ)</t>
-        </is>
-      </c>
+      <c r="B45" s="60" t="inlineStr">
+        <is>
+          <t>Rule 4</t>
+        </is>
+      </c>
+      <c r="C45" s="61" t="inlineStr">
+        <is>
+          <t>8+ consecutive points on same side of CL</t>
+        </is>
+      </c>
+      <c r="D45" s="61" t="inlineStr">
+        <is>
+          <t>Mean has shifted</t>
+        </is>
+      </c>
+      <c r="E45" s="61" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="B46" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  8σ Spread — Contains ~99.9937% of process output (±4σ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="58" t="inlineStr"/>
+      <c r="B46" s="60" t="inlineStr">
+        <is>
+          <t>Rule 5</t>
+        </is>
+      </c>
+      <c r="C46" s="61" t="inlineStr">
+        <is>
+          <t>6 consecutive points trending up or down</t>
+        </is>
+      </c>
+      <c r="D46" s="61" t="inlineStr">
+        <is>
+          <t>Drift (tool wear, temp)</t>
+        </is>
+      </c>
+      <c r="E46" s="61" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="B48" s="59" t="inlineStr">
-        <is>
-          <t>Color Coding</t>
+      <c r="B48" s="58" t="inlineStr">
+        <is>
+          <t>🏭 Industry Standard Requirements</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🟢 Green cells = Good / Capable / Within target</t>
-        </is>
-      </c>
+      <c r="B49" s="59" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="C49" s="59" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D49" s="59" t="inlineStr">
+        <is>
+          <t>Cpk Requirement</t>
+        </is>
+      </c>
+      <c r="E49" s="59" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="B50" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🟡 Yellow cells = Warning / Marginal</t>
-        </is>
-      </c>
+      <c r="B50" s="60" t="inlineStr">
+        <is>
+          <t>IATF 16949</t>
+        </is>
+      </c>
+      <c r="C50" s="61" t="inlineStr">
+        <is>
+          <t>Automotive production</t>
+        </is>
+      </c>
+      <c r="D50" s="61" t="inlineStr">
+        <is>
+          <t>≥ 1.33 (ongoing), ≥ 1.67 (new)</t>
+        </is>
+      </c>
+      <c r="E50" s="61" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="B51" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🔴 Red cells = Bad / Action Required / Not capable</t>
-        </is>
-      </c>
+      <c r="B51" s="60" t="inlineStr">
+        <is>
+          <t>VDA 6.1</t>
+        </is>
+      </c>
+      <c r="C51" s="61" t="inlineStr">
+        <is>
+          <t>German automotive</t>
+        </is>
+      </c>
+      <c r="D51" s="61" t="inlineStr">
+        <is>
+          <t>≥ 1.33 (Cmk), ≥ 1.67 (critical)</t>
+        </is>
+      </c>
+      <c r="E51" s="61" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="B52" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🔵 Blue cells = Input cells (enter your data here)</t>
+      <c r="B52" s="60" t="inlineStr">
+        <is>
+          <t>AS9100</t>
+        </is>
+      </c>
+      <c r="C52" s="61" t="inlineStr">
+        <is>
+          <t>Aerospace</t>
+        </is>
+      </c>
+      <c r="D52" s="61" t="inlineStr">
+        <is>
+          <t>≥ 1.33 (typical), ≥ 1.5 (critical)</t>
+        </is>
+      </c>
+      <c r="E52" s="61" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="60" t="inlineStr">
+        <is>
+          <t>ISO 13485</t>
+        </is>
+      </c>
+      <c r="C53" s="61" t="inlineStr">
+        <is>
+          <t>Medical devices</t>
+        </is>
+      </c>
+      <c r="D53" s="61" t="inlineStr">
+        <is>
+          <t>≥ 1.33 (critical features)</t>
+        </is>
+      </c>
+      <c r="E53" s="61" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="B54" s="60" t="inlineStr">
+        <is>
+          <t>Six Sigma</t>
+        </is>
+      </c>
+      <c r="C54" s="61" t="inlineStr">
+        <is>
+          <t>General manufacturing</t>
+        </is>
+      </c>
+      <c r="D54" s="61" t="inlineStr">
+        <is>
+          <t>≥ 2.0 (6σ target)</t>
+        </is>
+      </c>
+      <c r="E54" s="61" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="B55" s="60" t="inlineStr">
+        <is>
+          <t>ISO 22514</t>
+        </is>
+      </c>
+      <c r="C55" s="61" t="inlineStr">
+        <is>
+          <t>Capability study std</t>
+        </is>
+      </c>
+      <c r="D55" s="61" t="inlineStr">
+        <is>
+          <t>Defines Cm/Cmk/Pp/Ppk procedures</t>
+        </is>
+      </c>
+      <c r="E55" s="61" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="58" t="inlineStr">
+        <is>
+          <t>📖 How to Use This Workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="62" t="inlineStr">
+        <is>
+          <t>1. Enter specifications (Tₘ, LSL, USL) in the Analysis sheet (blue cells)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="62" t="inlineStr">
+        <is>
+          <t>2. Choose Mode: 'Enter Manually' or 'Use Data Worksheet' (dropdown in C10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="62" t="inlineStr">
+        <is>
+          <t>3. If Manual: enter x̄, σ, n directly in the Analysis sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="62" t="inlineStr">
+        <is>
+          <t>4. If Worksheet: enter part data in the Data sheet — mean &amp; σ auto-link</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="62" t="inlineStr">
+        <is>
+          <t>5. All results, probability, hypothesis test, and verdict update INSTANTLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="62" t="inlineStr">
+        <is>
+          <t>6. View charts in the Charts sheet (I-MR control chart, bell curve, capability bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="62" t="inlineStr">
+        <is>
+          <t>7. To save a run: go to History sheet, copy Row 4, paste as VALUES into Row 5+</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="58" t="inlineStr">
+        <is>
+          <t>🎨 Color Coding</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="63" t="inlineStr">
+        <is>
+          <t>🟢 Green cells</t>
+        </is>
+      </c>
+      <c r="C67" s="64" t="inlineStr">
+        <is>
+          <t>Good / Capable / Within target</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="63" t="inlineStr">
+        <is>
+          <t>🟡 Yellow cells</t>
+        </is>
+      </c>
+      <c r="C68" s="64" t="inlineStr">
+        <is>
+          <t>Warning / Marginal</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="63" t="inlineStr">
+        <is>
+          <t>🔴 Red cells</t>
+        </is>
+      </c>
+      <c r="C69" s="64" t="inlineStr">
+        <is>
+          <t>Bad / Action Required / Not capable</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="63" t="inlineStr">
+        <is>
+          <t>🔵 Blue cells</t>
+        </is>
+      </c>
+      <c r="C70" s="64" t="inlineStr">
+        <is>
+          <t>Input cells (enter your data here)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="B66:E66"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>